<commit_message>
clean up imports and requirements
</commit_message>
<xml_diff>
--- a/lib/onc_certification_g33_test_kit/requirements/170.315(g)(33)_HTI-4_requirements.xlsx
+++ b/lib/onc_certification_g33_test_kit/requirements/170.315(g)(33)_HTI-4_requirements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/knaden/Documents/Inferno/source/inferno-core/lib/inferno/apps/cli/templates/lib/%library_name%/requirements/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/onc-certification-g33-test-kit/lib/onc_certification_g33_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD601077-115E-444F-9487-4C7E8CBC653D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8967BFCA-9B43-8E4A-A3A3-9E9E8C0F8A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" firstSheet="1" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="33820" windowHeight="20640" firstSheet="1" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="9" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="146">
   <si>
     <t>General Information</t>
   </si>
@@ -385,76 +385,40 @@
     <t>170.315(g)(33)</t>
   </si>
   <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6075</t>
-  </si>
-  <si>
-    <t>Support submitting a prior authorization request as a client in accordance with at least one of the versions of the implementation specification adopted in § 170.215(j)(3) [([*Prior authorization submission*](https://www.federalregister.gov/d/2025-14681/p-5994)) currently including only [PAS 2.0.1](https://hl7.org/fhir/us/davinci-pas/STU2/)]</t>
-  </si>
-  <si>
     <t>170.315(g)(33)(i)</t>
   </si>
   <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6076</t>
-  </si>
-  <si>
     <t>Support registration capabilities applicable to a client system.</t>
   </si>
   <si>
     <t>170.315(g)(33)(i)(A)</t>
   </si>
   <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6077</t>
-  </si>
-  <si>
-    <t>Support system authentication and authorization as a client in accordance with the “Backend Services” section of at least one of the versions of the implementation specification adopted in § 170.215(c) [([*Application access and launch*](https://www.federalregister.gov/d/2025-14681/p-5973)) currently including SMART App Launch versions [1.0.0](https://hl7.org/fhir/smart-app-launch/1.0.0/) and [2.0.0](https://hl7.org/fhir/smart-app-launch/STU2/)].</t>
-  </si>
-  <si>
     <t>170.315(g)(33)(i)(B)</t>
   </si>
   <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6078</t>
-  </si>
-  <si>
     <t>Support the ability to submit a prior authorization request as a client system</t>
   </si>
   <si>
     <t>170.315(g)(33)(i)(C)</t>
   </si>
   <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6079</t>
-  </si>
-  <si>
     <t>Support the capabilities in the “EHR PAS Capabilities” Capability Statement.</t>
   </si>
   <si>
     <t>170.315(g)(33)(i)(C)(1)</t>
   </si>
   <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6080</t>
-  </si>
-  <si>
     <t>Support the ability to consume and process a “ClaimResponse.”</t>
   </si>
   <si>
     <t>170.315(g)(33)(i)(C)(2)</t>
   </si>
   <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6081</t>
-  </si>
-  <si>
-    <t>Support subscriptions as a client according to the requirements in paragraph (j)(21) [([*Subscriptions—client*](https://www.federalregister.gov/d/2025-14681/p-6095))] of this section in order to support “pended authorization responses.”</t>
-  </si>
-  <si>
     <t>170.315(j)(21)_HTI-4#Client</t>
   </si>
   <si>
     <t>170.315(g)(33)(i)(C)(3)</t>
-  </si>
-  <si>
-    <t>https://www.federalregister.gov/d/2025-14681/p-6082</t>
-  </si>
-  <si>
-    <t>Supported subscriptions client endpoint capabilities for the “REST-Hook” channel from implementation specifications adopted in § 170.215(j)(3)  [([*Prior authorization submission*](https://www.federalregister.gov/d/2025-14681/p-5994)) currently including only [PAS 2.0.1](https://hl7.org/fhir/us/davinci-pas/STU2/)] must include complete accompanying technical documentation.</t>
   </si>
   <si>
     <t>170.315(g)(33)(ii)</t>
@@ -798,12 +762,51 @@
   <si>
     <t>DEPRECATED</t>
   </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(i)</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(i)(A)</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(i)(B)</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(i)©</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(i)(C)(1)</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(i)(C)(2)</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(i)(C)(3)</t>
+  </si>
+  <si>
+    <t>https://www.ecfr.gov/current/title-45/part-170/section-170.315#p-170.315(g)(33)(ii)</t>
+  </si>
+  <si>
+    <t>Supported subscriptions client endpoint capabilities for the “REST-Hook” channel from implementation specifications adopted in § [170.215(j)(3)](https://www.ecfr.gov/current/title-45/part-170/section-170.215#p-170.215(j)(3)) must include complete accompanying technical documentation.</t>
+  </si>
+  <si>
+    <t>Support subscriptions as a client according to the requirements in [paragraph (j)(21)](https://www.ecfr.gov/current/title-45/section-170.315#p-170.315(j)(21)) of this section in order to support “pended authorization responses.”</t>
+  </si>
+  <si>
+    <t>Support system authentication and authorization as a client in accordance with the “Backend Services” section of at least one of the versions of the implementation specification adopted in [§ 170.215](https://www.ecfr.gov/current/title-45/section-170.215#p-170.215(c)).</t>
+  </si>
+  <si>
+    <t>Support submitting a prior authorization request as a client in accordance with at least one of the versions of the implementation specification adopted in [§ 170.215(j)(3)](https://www.ecfr.gov/current/title-45/section-170.215#p-170.215(j)(3))</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1109,6 +1112,15 @@
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1117,15 +1129,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1466,16 +1469,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6AA7094-ECFF-0B4E-A5C9-6F41B8D76EEB}">
   <dimension ref="A1:D38"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.375" style="15" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" style="15" customWidth="1"/>
     <col min="2" max="2" width="133.5" style="20" customWidth="1"/>
     <col min="3" max="3" width="52.5" style="20" customWidth="1"/>
-    <col min="4" max="4" width="91.125" style="20" customWidth="1"/>
-    <col min="5" max="16384" width="10.875" style="15"/>
+    <col min="4" max="4" width="91.1640625" style="20" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21.95" customHeight="1">
+    <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
@@ -1483,47 +1486,47 @@
       <c r="C1" s="34"/>
       <c r="D1" s="15"/>
     </row>
-    <row r="2" spans="1:4" ht="51" customHeight="1">
+    <row r="2" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="35"/>
+      <c r="C2" s="38"/>
       <c r="D2" s="15"/>
     </row>
-    <row r="3" spans="1:4" ht="33.950000000000003">
+    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="36"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="15"/>
     </row>
-    <row r="4" spans="1:4" ht="80.099999999999994" customHeight="1">
+    <row r="4" spans="1:4" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="36"/>
+      <c r="C4" s="39"/>
       <c r="D4" s="15"/>
     </row>
-    <row r="5" spans="1:4" ht="63.95" customHeight="1">
+    <row r="5" spans="1:4" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="37"/>
+      <c r="C5" s="40"/>
       <c r="D5" s="15"/>
     </row>
-    <row r="6" spans="1:4" ht="21.95" customHeight="1">
+    <row r="6" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34" t="s">
         <v>9</v>
       </c>
@@ -1531,57 +1534,57 @@
       <c r="C6" s="34"/>
       <c r="D6" s="15"/>
     </row>
-    <row r="7" spans="1:4" ht="17.100000000000001">
+    <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="36"/>
+      <c r="C7" s="39"/>
       <c r="D7" s="15"/>
     </row>
-    <row r="8" spans="1:4" ht="33.950000000000003">
+    <row r="8" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="36"/>
+      <c r="C8" s="39"/>
       <c r="D8" s="15"/>
     </row>
-    <row r="9" spans="1:4" ht="32.1" customHeight="1">
+    <row r="9" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="36"/>
+      <c r="C9" s="39"/>
       <c r="D9" s="15"/>
     </row>
-    <row r="10" spans="1:4" ht="33.950000000000003">
+    <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="36"/>
+      <c r="C10" s="39"/>
       <c r="D10" s="15"/>
     </row>
-    <row r="11" spans="1:4" ht="32.1" customHeight="1">
+    <row r="11" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="36"/>
+      <c r="C11" s="39"/>
       <c r="D11" s="15"/>
     </row>
-    <row r="12" spans="1:4" ht="21.95" customHeight="1">
+    <row r="12" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="34" t="s">
         <v>20</v>
       </c>
@@ -1589,7 +1592,7 @@
       <c r="C12" s="34"/>
       <c r="D12" s="15"/>
     </row>
-    <row r="13" spans="1:4" ht="17.100000000000001">
+    <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="s">
         <v>21</v>
       </c>
@@ -1601,7 +1604,7 @@
       </c>
       <c r="D13" s="15"/>
     </row>
-    <row r="14" spans="1:4" ht="32.1">
+    <row r="14" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A14" s="29" t="s">
         <v>24</v>
       </c>
@@ -1613,7 +1616,7 @@
       </c>
       <c r="D14" s="23"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="29" t="s">
         <v>27</v>
       </c>
@@ -1625,7 +1628,7 @@
       </c>
       <c r="D15" s="21"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="29" t="s">
         <v>30</v>
       </c>
@@ -1637,7 +1640,7 @@
       </c>
       <c r="D16" s="21"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="29" t="s">
         <v>33</v>
       </c>
@@ -1649,7 +1652,7 @@
       </c>
       <c r="D17" s="21"/>
     </row>
-    <row r="18" spans="1:4" ht="32.1">
+    <row r="18" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="29" t="s">
         <v>36</v>
       </c>
@@ -1661,7 +1664,7 @@
       </c>
       <c r="D18" s="21"/>
     </row>
-    <row r="19" spans="1:4" ht="111.95">
+    <row r="19" spans="1:4" ht="112" x14ac:dyDescent="0.2">
       <c r="A19" s="29" t="s">
         <v>39</v>
       </c>
@@ -1673,7 +1676,7 @@
       </c>
       <c r="D19" s="21"/>
     </row>
-    <row r="20" spans="1:4" ht="32.1">
+    <row r="20" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="29" t="s">
         <v>42</v>
       </c>
@@ -1685,7 +1688,7 @@
       </c>
       <c r="D20" s="21"/>
     </row>
-    <row r="21" spans="1:4" ht="32.1">
+    <row r="21" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="30" t="s">
         <v>45</v>
       </c>
@@ -1697,7 +1700,7 @@
       </c>
       <c r="D21" s="21"/>
     </row>
-    <row r="22" spans="1:4" ht="32.1">
+    <row r="22" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="29" t="s">
         <v>48</v>
       </c>
@@ -1709,7 +1712,7 @@
       </c>
       <c r="D22" s="21"/>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="29" t="s">
         <v>50</v>
       </c>
@@ -1721,7 +1724,7 @@
       </c>
       <c r="D23" s="21"/>
     </row>
-    <row r="24" spans="1:4" ht="32.1">
+    <row r="24" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="29" t="s">
         <v>52</v>
       </c>
@@ -1733,7 +1736,7 @@
       </c>
       <c r="D24" s="21"/>
     </row>
-    <row r="25" spans="1:4" ht="32.1">
+    <row r="25" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="29" t="s">
         <v>54</v>
       </c>
@@ -1745,7 +1748,7 @@
       </c>
       <c r="D25" s="21"/>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="31" t="s">
         <v>56</v>
       </c>
@@ -1756,7 +1759,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="31" t="s">
         <v>58</v>
       </c>
@@ -1767,7 +1770,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="68.099999999999994" customHeight="1">
+    <row r="28" spans="1:4" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="30" t="s">
         <v>60</v>
       </c>
@@ -1778,7 +1781,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="30" t="s">
         <v>62</v>
       </c>
@@ -1790,7 +1793,7 @@
       </c>
       <c r="D29" s="15"/>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="30" t="s">
         <v>64</v>
       </c>
@@ -1802,7 +1805,7 @@
       </c>
       <c r="D30" s="15"/>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="30" t="s">
         <v>66</v>
       </c>
@@ -1814,7 +1817,7 @@
       </c>
       <c r="D31" s="15"/>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="30" t="s">
         <v>68</v>
       </c>
@@ -1826,7 +1829,7 @@
       </c>
       <c r="D32" s="15"/>
     </row>
-    <row r="33" spans="1:4" ht="32.1">
+    <row r="33" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="30" t="s">
         <v>70</v>
       </c>
@@ -1838,7 +1841,7 @@
       </c>
       <c r="D33" s="15"/>
     </row>
-    <row r="34" spans="1:4" ht="21.95">
+    <row r="34" spans="1:4" ht="22" x14ac:dyDescent="0.3">
       <c r="A34" s="34" t="s">
         <v>72</v>
       </c>
@@ -1846,51 +1849,46 @@
       <c r="C34" s="34"/>
       <c r="D34" s="15"/>
     </row>
-    <row r="35" spans="1:4" ht="48" customHeight="1">
+    <row r="35" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="38" t="s">
+      <c r="B35" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="38"/>
-    </row>
-    <row r="36" spans="1:4" ht="134.1" customHeight="1">
+      <c r="C35" s="35"/>
+    </row>
+    <row r="36" spans="1:4" ht="134" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="B36" s="39" t="s">
+      <c r="B36" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="C36" s="40"/>
-    </row>
-    <row r="37" spans="1:4" ht="111.95" customHeight="1">
+      <c r="C36" s="37"/>
+    </row>
+    <row r="37" spans="1:4" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="B37" s="38" t="s">
+      <c r="B37" s="35" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="38"/>
+      <c r="C37" s="35"/>
       <c r="D37" s="15"/>
     </row>
-    <row r="38" spans="1:4" ht="48" customHeight="1">
+    <row r="38" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="B38" s="38" t="s">
+      <c r="B38" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="C38" s="38"/>
+      <c r="C38" s="35"/>
       <c r="D38" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B36:C36"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="B2:C2"/>
@@ -1903,6 +1901,11 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B36:C36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1911,33 +1914,33 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0272D98A-080C-3945-A7E0-CB54FB3A65A9}">
   <dimension ref="A1:AJ346"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.875" style="7"/>
+    <col min="1" max="2" width="10.83203125" style="7"/>
     <col min="3" max="3" width="41" style="8" customWidth="1"/>
-    <col min="4" max="4" width="13.375" style="7" customWidth="1"/>
-    <col min="5" max="5" width="10.875" style="7"/>
-    <col min="6" max="6" width="13.375" style="8" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" style="7"/>
+    <col min="6" max="6" width="13.33203125" style="8" customWidth="1"/>
     <col min="7" max="7" width="14" style="7" customWidth="1"/>
-    <col min="8" max="8" width="24.625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="24.6640625" style="10" customWidth="1"/>
     <col min="9" max="9" width="10" style="8" customWidth="1"/>
     <col min="10" max="10" width="22" style="8" customWidth="1"/>
     <col min="11" max="11" width="10.5" style="8" customWidth="1"/>
-    <col min="12" max="12" width="25.875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" style="8" customWidth="1"/>
     <col min="13" max="13" width="20" style="9" customWidth="1"/>
     <col min="14" max="14" width="28.5" style="9" customWidth="1"/>
-    <col min="15" max="16" width="10.875" style="10"/>
+    <col min="15" max="16" width="10.83203125" style="10"/>
     <col min="17" max="17" width="10.5" style="16" customWidth="1"/>
     <col min="18" max="18" width="42.5" style="10" customWidth="1"/>
-    <col min="19" max="20" width="44.125" style="10" customWidth="1"/>
-    <col min="21" max="21" width="10.875" style="6"/>
+    <col min="19" max="20" width="44.1640625" style="10" customWidth="1"/>
+    <col min="21" max="21" width="10.83203125" style="6"/>
     <col min="22" max="22" width="11" style="6" customWidth="1"/>
-    <col min="23" max="24" width="10.875" style="6"/>
-    <col min="25" max="25" width="14.875" style="6" customWidth="1"/>
-    <col min="26" max="16384" width="10.875" style="6"/>
+    <col min="23" max="24" width="10.83203125" style="6"/>
+    <col min="25" max="25" width="14.83203125" style="6" customWidth="1"/>
+    <col min="26" max="16384" width="10.83203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="5" customFormat="1" ht="32.1">
+    <row r="1" spans="1:36" s="5" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2001,12 +2004,12 @@
       <c r="U1" s="6"/>
       <c r="Z1" s="6"/>
     </row>
-    <row r="2" spans="1:36" ht="30.75">
+    <row r="2" spans="1:36" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="7">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>84</v>
+        <v>133</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>85</v>
@@ -2023,7 +2026,7 @@
       </c>
       <c r="N2" s="9" t="str" cm="1">
         <f t="array" ref="N2">SECTION_NAME(B2)</f>
-        <v/>
+        <v>p-170.315(g)(33)</v>
       </c>
       <c r="O2" s="10" t="s">
         <v>88</v>
@@ -2039,15 +2042,15 @@
       <c r="AI2" s="5"/>
       <c r="AJ2" s="5"/>
     </row>
-    <row r="3" spans="1:36" ht="120.75" customHeight="1">
+    <row r="3" spans="1:36" ht="120.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7">
         <v>2</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>89</v>
+        <v>134</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>86</v>
@@ -2061,10 +2064,10 @@
       </c>
       <c r="N3" s="9" t="str" cm="1">
         <f t="array" ref="N3">SECTION_NAME(B3)</f>
-        <v/>
+        <v>p-170.315(g)(33)(i)</v>
       </c>
       <c r="O3" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="Z3" s="13"/>
       <c r="AA3" s="5"/>
@@ -2074,15 +2077,15 @@
       <c r="AE3" s="5"/>
       <c r="AF3" s="5"/>
     </row>
-    <row r="4" spans="1:36" ht="30.75">
+    <row r="4" spans="1:36" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="7">
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>92</v>
+        <v>135</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>86</v>
@@ -2096,10 +2099,10 @@
       </c>
       <c r="N4" s="9" t="str" cm="1">
         <f t="array" ref="N4">SECTION_NAME(B4)</f>
-        <v/>
+        <v>p-170.315(g)(33)(i)(A)</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="Z4" s="13"/>
       <c r="AA4" s="5"/>
@@ -2109,15 +2112,15 @@
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
     </row>
-    <row r="5" spans="1:36" ht="207.75" customHeight="1">
+    <row r="5" spans="1:36" ht="207.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7">
         <v>4</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>95</v>
+        <v>136</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>86</v>
@@ -2131,10 +2134,10 @@
       </c>
       <c r="N5" s="9" t="str" cm="1">
         <f t="array" ref="N5">SECTION_NAME(B5)</f>
-        <v/>
+        <v>p-170.315(g)(33)(i)(B)</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="Z5" s="13"/>
       <c r="AA5" s="5"/>
@@ -2144,15 +2147,15 @@
       <c r="AE5" s="5"/>
       <c r="AF5" s="5"/>
     </row>
-    <row r="6" spans="1:36" ht="30.75">
+    <row r="6" spans="1:36" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="7">
         <v>5</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>86</v>
@@ -2166,10 +2169,10 @@
       </c>
       <c r="N6" s="9" t="str" cm="1">
         <f t="array" ref="N6">SECTION_NAME(B6)</f>
-        <v/>
+        <v>p-170.315(g)(33)(i)©</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="Y6" s="14"/>
       <c r="Z6" s="13"/>
@@ -2180,15 +2183,15 @@
       <c r="AE6" s="5"/>
       <c r="AF6" s="5"/>
     </row>
-    <row r="7" spans="1:36" ht="30.75">
+    <row r="7" spans="1:36" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="7">
         <v>6</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>101</v>
+        <v>138</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>86</v>
@@ -2202,21 +2205,21 @@
       </c>
       <c r="N7" s="9" t="str" cm="1">
         <f t="array" ref="N7">SECTION_NAME(B7)</f>
-        <v/>
+        <v>p-170.315(g)(33)(i)(C)(1)</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="8" spans="1:36" ht="30.75">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:36" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="7">
         <v>7</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>104</v>
+        <v>139</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>86</v>
@@ -2230,21 +2233,21 @@
       </c>
       <c r="N8" s="9" t="str" cm="1">
         <f t="array" ref="N8">SECTION_NAME(B8)</f>
-        <v/>
+        <v>p-170.315(g)(33)(i)(C)(2)</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="9" spans="1:36" ht="121.5" customHeight="1">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" ht="121.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7">
         <v>8</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>107</v>
+        <v>140</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>86</v>
@@ -2253,7 +2256,7 @@
         <v>87</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="M9" s="9" t="str" cm="1">
         <f t="array" ref="M9">PAGE_NAME(B9)</f>
@@ -2261,21 +2264,21 @@
       </c>
       <c r="N9" s="9" t="str" cm="1">
         <f t="array" ref="N9">SECTION_NAME(B9)</f>
-        <v/>
+        <v>p-170.315(g)(33)(i)(C)(3)</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:36" ht="154.5" customHeight="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:36" ht="154.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="7">
         <v>9</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>86</v>
@@ -2289,13 +2292,13 @@
       </c>
       <c r="N10" s="9" t="str" cm="1">
         <f t="array" ref="N10">SECTION_NAME(B10)</f>
-        <v/>
+        <v>p-170.315(g)(33)(ii)</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:36" ht="15.95">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:36" ht="16" x14ac:dyDescent="0.2">
       <c r="M11" s="9" t="str" cm="1">
         <f t="array" ref="M11">PAGE_NAME(B11)</f>
         <v/>
@@ -2305,7 +2308,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:36" ht="15.95">
+    <row r="12" spans="1:36" ht="16" x14ac:dyDescent="0.2">
       <c r="M12" s="9" t="str" cm="1">
         <f t="array" ref="M12">PAGE_NAME(B12)</f>
         <v/>
@@ -2315,7 +2318,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:36" ht="15.95">
+    <row r="13" spans="1:36" ht="16" x14ac:dyDescent="0.2">
       <c r="M13" s="9" t="str" cm="1">
         <f t="array" ref="M13">PAGE_NAME(B13)</f>
         <v/>
@@ -2325,7 +2328,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:36" ht="15.95">
+    <row r="14" spans="1:36" ht="16" x14ac:dyDescent="0.2">
       <c r="M14" s="9" t="str" cm="1">
         <f t="array" ref="M14">PAGE_NAME(B14)</f>
         <v/>
@@ -2335,7 +2338,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:36" ht="15.95">
+    <row r="15" spans="1:36" ht="16" x14ac:dyDescent="0.2">
       <c r="M15" s="9" t="str" cm="1">
         <f t="array" ref="M15">PAGE_NAME(B15)</f>
         <v/>
@@ -2345,7 +2348,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:36" ht="15.95">
+    <row r="16" spans="1:36" ht="16" x14ac:dyDescent="0.2">
       <c r="M16" s="9" t="str" cm="1">
         <f t="array" ref="M16">PAGE_NAME(B16)</f>
         <v/>
@@ -2355,7 +2358,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="13:18" ht="15.95">
+    <row r="17" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M17" s="9" t="str" cm="1">
         <f t="array" ref="M17">PAGE_NAME(B17)</f>
         <v/>
@@ -2365,7 +2368,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="13:18" ht="15.95">
+    <row r="18" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M18" s="9" t="str" cm="1">
         <f t="array" ref="M18">PAGE_NAME(B18)</f>
         <v/>
@@ -2375,7 +2378,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="13:18" ht="15.95">
+    <row r="19" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M19" s="9" t="str" cm="1">
         <f t="array" ref="M19">PAGE_NAME(B19)</f>
         <v/>
@@ -2385,7 +2388,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="13:18" ht="15.95">
+    <row r="20" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M20" s="9" t="str" cm="1">
         <f t="array" ref="M20">PAGE_NAME(B20)</f>
         <v/>
@@ -2396,7 +2399,7 @@
       </c>
       <c r="R20" s="16"/>
     </row>
-    <row r="21" spans="13:18" ht="15.95">
+    <row r="21" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M21" s="9" t="str" cm="1">
         <f t="array" ref="M21">PAGE_NAME(B21)</f>
         <v/>
@@ -2406,7 +2409,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="13:18" ht="15.95">
+    <row r="22" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M22" s="9" t="str" cm="1">
         <f t="array" ref="M22">PAGE_NAME(B22)</f>
         <v/>
@@ -2416,7 +2419,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="13:18" ht="15.95">
+    <row r="23" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M23" s="9" t="str" cm="1">
         <f t="array" ref="M23">PAGE_NAME(B23)</f>
         <v/>
@@ -2426,7 +2429,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="13:18" ht="15.95">
+    <row r="24" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M24" s="9" t="str" cm="1">
         <f t="array" ref="M24">PAGE_NAME(B24)</f>
         <v/>
@@ -2436,7 +2439,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="13:18" ht="15.95">
+    <row r="25" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M25" s="9" t="str" cm="1">
         <f t="array" ref="M25">PAGE_NAME(B25)</f>
         <v/>
@@ -2446,7 +2449,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="13:18" ht="15.95">
+    <row r="26" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M26" s="9" t="str" cm="1">
         <f t="array" ref="M26">PAGE_NAME(B26)</f>
         <v/>
@@ -2456,7 +2459,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="13:18" ht="15.95">
+    <row r="27" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M27" s="9" t="str" cm="1">
         <f t="array" ref="M27">PAGE_NAME(B27)</f>
         <v/>
@@ -2466,7 +2469,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="13:18" ht="15.95">
+    <row r="28" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M28" s="9" t="str" cm="1">
         <f t="array" ref="M28">PAGE_NAME(B28)</f>
         <v/>
@@ -2476,7 +2479,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="13:18" ht="15.95">
+    <row r="29" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M29" s="9" t="str" cm="1">
         <f t="array" ref="M29">PAGE_NAME(B29)</f>
         <v/>
@@ -2486,7 +2489,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="13:18" ht="15.95">
+    <row r="30" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M30" s="9" t="str" cm="1">
         <f t="array" ref="M30">PAGE_NAME(B30)</f>
         <v/>
@@ -2496,7 +2499,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="13:18" ht="15.95">
+    <row r="31" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M31" s="9" t="str" cm="1">
         <f t="array" ref="M31">PAGE_NAME(B31)</f>
         <v/>
@@ -2506,7 +2509,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="13:18" ht="15.95">
+    <row r="32" spans="13:18" ht="16" x14ac:dyDescent="0.2">
       <c r="M32" s="9" t="str" cm="1">
         <f t="array" ref="M32">PAGE_NAME(B32)</f>
         <v/>
@@ -2516,7 +2519,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="2:14" ht="15.95">
+    <row r="33" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M33" s="9" t="str" cm="1">
         <f t="array" ref="M33">PAGE_NAME(B33)</f>
         <v/>
@@ -2526,7 +2529,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="2:14" ht="15.95">
+    <row r="34" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M34" s="9" t="str" cm="1">
         <f t="array" ref="M34">PAGE_NAME(B34)</f>
         <v/>
@@ -2536,7 +2539,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="2:14" ht="15.95">
+    <row r="35" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M35" s="9" t="str" cm="1">
         <f t="array" ref="M35">PAGE_NAME(B35)</f>
         <v/>
@@ -2546,7 +2549,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="2:14" ht="15.95">
+    <row r="36" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M36" s="9" t="str" cm="1">
         <f t="array" ref="M36">PAGE_NAME(B36)</f>
         <v/>
@@ -2556,7 +2559,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="2:14" ht="15.95">
+    <row r="37" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M37" s="9" t="str" cm="1">
         <f t="array" ref="M37">PAGE_NAME(B37)</f>
         <v/>
@@ -2566,7 +2569,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="2:14" ht="15.95">
+    <row r="38" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M38" s="9" t="str" cm="1">
         <f t="array" ref="M38">PAGE_NAME(B38)</f>
         <v/>
@@ -2576,7 +2579,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="2:14" ht="15.95">
+    <row r="39" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M39" s="9" t="str" cm="1">
         <f t="array" ref="M39">PAGE_NAME(B39)</f>
         <v/>
@@ -2586,7 +2589,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="2:14" ht="15.95">
+    <row r="40" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M40" s="9" t="str" cm="1">
         <f t="array" ref="M40">PAGE_NAME(B40)</f>
         <v/>
@@ -2596,7 +2599,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="2:14" ht="15.95">
+    <row r="41" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M41" s="9" t="str" cm="1">
         <f t="array" ref="M41">PAGE_NAME(B41)</f>
         <v/>
@@ -2606,7 +2609,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="2:14" ht="15.95">
+    <row r="42" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M42" s="9" t="str" cm="1">
         <f t="array" ref="M42">PAGE_NAME(B42)</f>
         <v/>
@@ -2616,7 +2619,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="2:14" ht="15.95">
+    <row r="43" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M43" s="9" t="str" cm="1">
         <f t="array" ref="M43">PAGE_NAME(B43)</f>
         <v/>
@@ -2626,7 +2629,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="2:14" ht="15.95">
+    <row r="44" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M44" s="9" t="str" cm="1">
         <f t="array" ref="M44">PAGE_NAME(B44)</f>
         <v/>
@@ -2636,7 +2639,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="2:14" ht="15.95">
+    <row r="45" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M45" s="9" t="str" cm="1">
         <f t="array" ref="M45">PAGE_NAME(B45)</f>
         <v/>
@@ -2646,7 +2649,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="2:14" ht="15.95">
+    <row r="46" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B46" s="11"/>
       <c r="M46" s="9" t="str" cm="1">
         <f t="array" ref="M46">PAGE_NAME(B46)</f>
@@ -2657,7 +2660,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="2:14" ht="15.95">
+    <row r="47" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M47" s="9" t="str" cm="1">
         <f t="array" ref="M47">PAGE_NAME(B47)</f>
         <v/>
@@ -2667,7 +2670,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="2:14" ht="15.95">
+    <row r="48" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M48" s="9" t="str" cm="1">
         <f t="array" ref="M48">PAGE_NAME(B48)</f>
         <v/>
@@ -2677,7 +2680,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="13:14" ht="15.95">
+    <row r="49" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M49" s="9" t="str" cm="1">
         <f t="array" ref="M49">PAGE_NAME(B49)</f>
         <v/>
@@ -2687,7 +2690,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="13:14" ht="15.95">
+    <row r="50" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M50" s="9" t="str" cm="1">
         <f t="array" ref="M50">PAGE_NAME(B50)</f>
         <v/>
@@ -2697,7 +2700,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="13:14" ht="15.95">
+    <row r="51" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M51" s="9" t="str" cm="1">
         <f t="array" ref="M51">PAGE_NAME(B51)</f>
         <v/>
@@ -2707,7 +2710,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="13:14" ht="15.95">
+    <row r="52" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M52" s="9" t="str" cm="1">
         <f t="array" ref="M52">PAGE_NAME(B52)</f>
         <v/>
@@ -2717,7 +2720,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="13:14" ht="15.95">
+    <row r="53" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M53" s="9" t="str" cm="1">
         <f t="array" ref="M53">PAGE_NAME(B53)</f>
         <v/>
@@ -2727,7 +2730,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="13:14" ht="15.95">
+    <row r="54" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M54" s="9" t="str" cm="1">
         <f t="array" ref="M54">PAGE_NAME(B54)</f>
         <v/>
@@ -2737,7 +2740,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="13:14" ht="15.95">
+    <row r="55" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M55" s="9" t="str" cm="1">
         <f t="array" ref="M55">PAGE_NAME(B55)</f>
         <v/>
@@ -2747,7 +2750,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="13:14" ht="15.95">
+    <row r="56" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M56" s="9" t="str" cm="1">
         <f t="array" ref="M56">PAGE_NAME(B56)</f>
         <v/>
@@ -2757,7 +2760,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="13:14" ht="15.95">
+    <row r="57" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M57" s="9" t="str" cm="1">
         <f t="array" ref="M57">PAGE_NAME(B57)</f>
         <v/>
@@ -2767,7 +2770,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="13:14" ht="15.95">
+    <row r="58" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M58" s="9" t="str" cm="1">
         <f t="array" ref="M58">PAGE_NAME(B58)</f>
         <v/>
@@ -2777,7 +2780,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="13:14" ht="15.95">
+    <row r="59" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M59" s="9" t="str" cm="1">
         <f t="array" ref="M59">PAGE_NAME(B59)</f>
         <v/>
@@ -2787,7 +2790,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="13:14" ht="15.95">
+    <row r="60" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M60" s="9" t="str" cm="1">
         <f t="array" ref="M60">PAGE_NAME(B60)</f>
         <v/>
@@ -2797,7 +2800,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="13:14" ht="15.95">
+    <row r="61" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M61" s="9" t="str" cm="1">
         <f t="array" ref="M61">PAGE_NAME(B61)</f>
         <v/>
@@ -2807,7 +2810,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="13:14" ht="15.95">
+    <row r="62" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M62" s="9" t="str" cm="1">
         <f t="array" ref="M62">PAGE_NAME(B62)</f>
         <v/>
@@ -2817,7 +2820,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="13:14" ht="15.95">
+    <row r="63" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M63" s="9" t="str" cm="1">
         <f t="array" ref="M63">PAGE_NAME(B63)</f>
         <v/>
@@ -2827,7 +2830,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="13:14" ht="15.95">
+    <row r="64" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M64" s="9" t="str" cm="1">
         <f t="array" ref="M64">PAGE_NAME(B64)</f>
         <v/>
@@ -2837,7 +2840,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="13:14" ht="15.95">
+    <row r="65" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M65" s="9" t="str" cm="1">
         <f t="array" ref="M65">PAGE_NAME(B65)</f>
         <v/>
@@ -2847,7 +2850,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="13:14" ht="15.95">
+    <row r="66" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M66" s="9" t="str" cm="1">
         <f t="array" ref="M66">PAGE_NAME(B66)</f>
         <v/>
@@ -2857,7 +2860,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="13:14" ht="15.95">
+    <row r="67" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M67" s="9" t="str" cm="1">
         <f t="array" ref="M67">PAGE_NAME(B67)</f>
         <v/>
@@ -2867,7 +2870,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="13:14" ht="15.95">
+    <row r="68" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M68" s="9" t="str" cm="1">
         <f t="array" ref="M68">PAGE_NAME(B68)</f>
         <v/>
@@ -2877,7 +2880,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="13:14" ht="15.95">
+    <row r="69" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M69" s="9" t="str" cm="1">
         <f t="array" ref="M69">PAGE_NAME(B69)</f>
         <v/>
@@ -2887,7 +2890,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="13:14" ht="15.95">
+    <row r="70" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M70" s="9" t="str" cm="1">
         <f t="array" ref="M70">PAGE_NAME(B70)</f>
         <v/>
@@ -2897,7 +2900,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="13:14" ht="15.95">
+    <row r="71" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M71" s="9" t="str" cm="1">
         <f t="array" ref="M71">PAGE_NAME(B71)</f>
         <v/>
@@ -2907,7 +2910,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="13:14" ht="15.95">
+    <row r="72" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M72" s="9" t="str" cm="1">
         <f t="array" ref="M72">PAGE_NAME(B72)</f>
         <v/>
@@ -2917,7 +2920,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="13:14" ht="15.95">
+    <row r="73" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M73" s="9" t="str" cm="1">
         <f t="array" ref="M73">PAGE_NAME(B73)</f>
         <v/>
@@ -2927,7 +2930,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="13:14" ht="15.95">
+    <row r="74" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M74" s="9" t="str" cm="1">
         <f t="array" ref="M74">PAGE_NAME(B74)</f>
         <v/>
@@ -2937,7 +2940,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="13:14" ht="15.95">
+    <row r="75" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M75" s="9" t="str" cm="1">
         <f t="array" ref="M75">PAGE_NAME(B75)</f>
         <v/>
@@ -2947,7 +2950,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="13:14" ht="15.95">
+    <row r="76" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M76" s="9" t="str" cm="1">
         <f t="array" ref="M76">PAGE_NAME(B76)</f>
         <v/>
@@ -2957,7 +2960,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="13:14" ht="15.95">
+    <row r="77" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M77" s="9" t="str" cm="1">
         <f t="array" ref="M77">PAGE_NAME(B77)</f>
         <v/>
@@ -2967,7 +2970,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="13:14" ht="15.95">
+    <row r="78" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M78" s="9" t="str" cm="1">
         <f t="array" ref="M78">PAGE_NAME(B78)</f>
         <v/>
@@ -2977,7 +2980,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="13:14" ht="15.95">
+    <row r="79" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M79" s="9" t="str" cm="1">
         <f t="array" ref="M79">PAGE_NAME(B79)</f>
         <v/>
@@ -2987,7 +2990,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="13:14" ht="15.95">
+    <row r="80" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M80" s="9" t="str" cm="1">
         <f t="array" ref="M80">PAGE_NAME(B80)</f>
         <v/>
@@ -2997,7 +3000,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="6:14" ht="15.95">
+    <row r="81" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M81" s="9" t="str" cm="1">
         <f t="array" ref="M81">PAGE_NAME(B81)</f>
         <v/>
@@ -3007,7 +3010,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="6:14" ht="15.95">
+    <row r="82" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M82" s="9" t="str" cm="1">
         <f t="array" ref="M82">PAGE_NAME(B82)</f>
         <v/>
@@ -3017,7 +3020,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="6:14" ht="15.95">
+    <row r="83" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M83" s="9" t="str" cm="1">
         <f t="array" ref="M83">PAGE_NAME(B83)</f>
         <v/>
@@ -3027,7 +3030,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="6:14" ht="15.95">
+    <row r="84" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M84" s="9" t="str" cm="1">
         <f t="array" ref="M84">PAGE_NAME(B84)</f>
         <v/>
@@ -3037,7 +3040,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="6:14" ht="15.95">
+    <row r="85" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M85" s="9" t="str" cm="1">
         <f t="array" ref="M85">PAGE_NAME(B85)</f>
         <v/>
@@ -3047,7 +3050,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="6:14" ht="15.95">
+    <row r="86" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M86" s="9" t="str" cm="1">
         <f t="array" ref="M86">PAGE_NAME(B86)</f>
         <v/>
@@ -3057,7 +3060,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="6:14" ht="15.95">
+    <row r="87" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M87" s="9" t="str" cm="1">
         <f t="array" ref="M87">PAGE_NAME(B87)</f>
         <v/>
@@ -3067,7 +3070,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="6:14" ht="15.95">
+    <row r="88" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M88" s="9" t="str" cm="1">
         <f t="array" ref="M88">PAGE_NAME(B88)</f>
         <v/>
@@ -3077,7 +3080,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="6:14" ht="15.95">
+    <row r="89" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M89" s="9" t="str" cm="1">
         <f t="array" ref="M89">PAGE_NAME(B89)</f>
         <v/>
@@ -3087,7 +3090,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="6:14" ht="15.95">
+    <row r="90" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M90" s="9" t="str" cm="1">
         <f t="array" ref="M90">PAGE_NAME(B90)</f>
         <v/>
@@ -3097,7 +3100,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="6:14" ht="15.95">
+    <row r="91" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M91" s="9" t="str" cm="1">
         <f t="array" ref="M91">PAGE_NAME(B91)</f>
         <v/>
@@ -3107,7 +3110,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="6:14" ht="15.95">
+    <row r="92" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M92" s="9" t="str" cm="1">
         <f t="array" ref="M92">PAGE_NAME(B92)</f>
         <v/>
@@ -3117,7 +3120,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="6:14" ht="15.95">
+    <row r="93" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M93" s="9" t="str" cm="1">
         <f t="array" ref="M93">PAGE_NAME(B93)</f>
         <v/>
@@ -3127,7 +3130,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="6:14" ht="15.95">
+    <row r="94" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="F94" s="22"/>
       <c r="M94" s="9" t="str" cm="1">
         <f t="array" ref="M94">PAGE_NAME(B94)</f>
@@ -3138,7 +3141,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="6:14" ht="15.95">
+    <row r="95" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M95" s="9" t="str" cm="1">
         <f t="array" ref="M95">PAGE_NAME(B95)</f>
         <v/>
@@ -3148,7 +3151,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="6:14" ht="15.95">
+    <row r="96" spans="6:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M96" s="9" t="str" cm="1">
         <f t="array" ref="M96">PAGE_NAME(B96)</f>
         <v/>
@@ -3158,7 +3161,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:14" ht="15.95">
+    <row r="97" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A97" s="12"/>
       <c r="E97" s="12"/>
       <c r="M97" s="9" t="str" cm="1">
@@ -3170,7 +3173,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:14" ht="15.95">
+    <row r="98" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M98" s="9" t="str" cm="1">
         <f t="array" ref="M98">PAGE_NAME(B98)</f>
         <v/>
@@ -3180,7 +3183,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="1:14" ht="15.95">
+    <row r="99" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M99" s="9" t="str" cm="1">
         <f t="array" ref="M99">PAGE_NAME(B99)</f>
         <v/>
@@ -3190,7 +3193,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:14" ht="15.95">
+    <row r="100" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M100" s="9" t="str" cm="1">
         <f t="array" ref="M100">PAGE_NAME(B100)</f>
         <v/>
@@ -3200,7 +3203,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:14" ht="15.95">
+    <row r="101" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M101" s="9" t="str" cm="1">
         <f t="array" ref="M101">PAGE_NAME(B101)</f>
         <v/>
@@ -3210,7 +3213,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:14" ht="15.95">
+    <row r="102" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M102" s="9" t="str" cm="1">
         <f t="array" ref="M102">PAGE_NAME(B102)</f>
         <v/>
@@ -3220,7 +3223,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:14" ht="15.95">
+    <row r="103" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M103" s="9" t="str" cm="1">
         <f t="array" ref="M103">PAGE_NAME(B103)</f>
         <v/>
@@ -3230,7 +3233,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:14" ht="15.95">
+    <row r="104" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M104" s="9" t="str" cm="1">
         <f t="array" ref="M104">PAGE_NAME(B104)</f>
         <v/>
@@ -3240,7 +3243,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:14" ht="15.95">
+    <row r="105" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M105" s="9" t="str" cm="1">
         <f t="array" ref="M105">PAGE_NAME(B105)</f>
         <v/>
@@ -3250,7 +3253,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:14" ht="15.95">
+    <row r="106" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M106" s="9" t="str" cm="1">
         <f t="array" ref="M106">PAGE_NAME(B106)</f>
         <v/>
@@ -3260,7 +3263,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:14" ht="15.95">
+    <row r="107" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M107" s="9" t="str" cm="1">
         <f t="array" ref="M107">PAGE_NAME(B107)</f>
         <v/>
@@ -3270,7 +3273,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:14" ht="15.95">
+    <row r="108" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M108" s="9" t="str" cm="1">
         <f t="array" ref="M108">PAGE_NAME(B108)</f>
         <v/>
@@ -3280,7 +3283,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:14" ht="15.95">
+    <row r="109" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M109" s="9" t="str" cm="1">
         <f t="array" ref="M109">PAGE_NAME(B109)</f>
         <v/>
@@ -3290,7 +3293,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:14" ht="15.95">
+    <row r="110" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M110" s="9" t="str" cm="1">
         <f t="array" ref="M110">PAGE_NAME(B110)</f>
         <v/>
@@ -3300,7 +3303,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:14" ht="15.95">
+    <row r="111" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M111" s="9" t="str" cm="1">
         <f t="array" ref="M111">PAGE_NAME(B111)</f>
         <v/>
@@ -3310,7 +3313,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:14" ht="15.95">
+    <row r="112" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M112" s="9" t="str" cm="1">
         <f t="array" ref="M112">PAGE_NAME(B112)</f>
         <v/>
@@ -3320,7 +3323,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="9:17" ht="15.95">
+    <row r="113" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M113" s="9" t="str" cm="1">
         <f t="array" ref="M113">PAGE_NAME(B113)</f>
         <v/>
@@ -3330,7 +3333,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="9:17" ht="15.95">
+    <row r="114" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M114" s="9" t="str" cm="1">
         <f t="array" ref="M114">PAGE_NAME(B114)</f>
         <v/>
@@ -3340,7 +3343,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="9:17" ht="15.95">
+    <row r="115" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M115" s="9" t="str" cm="1">
         <f t="array" ref="M115">PAGE_NAME(B115)</f>
         <v/>
@@ -3350,7 +3353,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="9:17" ht="15.95">
+    <row r="116" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M116" s="9" t="str" cm="1">
         <f t="array" ref="M116">PAGE_NAME(B116)</f>
         <v/>
@@ -3360,7 +3363,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="9:17" ht="15.95">
+    <row r="117" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M117" s="9" t="str" cm="1">
         <f t="array" ref="M117">PAGE_NAME(B117)</f>
         <v/>
@@ -3370,7 +3373,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="9:17" ht="15.95">
+    <row r="118" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M118" s="9" t="str" cm="1">
         <f t="array" ref="M118">PAGE_NAME(B118)</f>
         <v/>
@@ -3380,7 +3383,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="9:17" ht="15.95">
+    <row r="119" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M119" s="9" t="str" cm="1">
         <f t="array" ref="M119">PAGE_NAME(B119)</f>
         <v/>
@@ -3390,7 +3393,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="9:17" ht="15.95">
+    <row r="120" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="I120" s="7"/>
       <c r="J120" s="7"/>
       <c r="K120" s="7"/>
@@ -3405,7 +3408,7 @@
       </c>
       <c r="Q120" s="10"/>
     </row>
-    <row r="121" spans="9:17" ht="15.95">
+    <row r="121" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M121" s="9" t="str" cm="1">
         <f t="array" ref="M121">PAGE_NAME(B121)</f>
         <v/>
@@ -3415,7 +3418,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="9:17" ht="15.95">
+    <row r="122" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M122" s="9" t="str" cm="1">
         <f t="array" ref="M122">PAGE_NAME(B122)</f>
         <v/>
@@ -3425,7 +3428,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="9:17" ht="15.95">
+    <row r="123" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M123" s="9" t="str" cm="1">
         <f t="array" ref="M123">PAGE_NAME(B123)</f>
         <v/>
@@ -3435,7 +3438,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="9:17" ht="15.95">
+    <row r="124" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M124" s="9" t="str" cm="1">
         <f t="array" ref="M124">PAGE_NAME(B124)</f>
         <v/>
@@ -3445,7 +3448,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="9:17" ht="15.95">
+    <row r="125" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M125" s="9" t="str" cm="1">
         <f t="array" ref="M125">PAGE_NAME(B125)</f>
         <v/>
@@ -3455,7 +3458,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="9:17" ht="15.95">
+    <row r="126" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M126" s="9" t="str" cm="1">
         <f t="array" ref="M126">PAGE_NAME(B126)</f>
         <v/>
@@ -3465,7 +3468,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="9:17" ht="15.95">
+    <row r="127" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M127" s="9" t="str" cm="1">
         <f t="array" ref="M127">PAGE_NAME(B127)</f>
         <v/>
@@ -3475,7 +3478,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="9:17" ht="15.95">
+    <row r="128" spans="9:17" ht="16" x14ac:dyDescent="0.2">
       <c r="M128" s="9" t="str" cm="1">
         <f t="array" ref="M128">PAGE_NAME(B128)</f>
         <v/>
@@ -3485,7 +3488,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="13:14" ht="15.95">
+    <row r="129" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M129" s="9" t="str" cm="1">
         <f t="array" ref="M129">PAGE_NAME(B129)</f>
         <v/>
@@ -3495,7 +3498,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="13:14" ht="15.95">
+    <row r="130" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M130" s="9" t="str" cm="1">
         <f t="array" ref="M130">PAGE_NAME(B130)</f>
         <v/>
@@ -3505,7 +3508,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="13:14" ht="15.95">
+    <row r="131" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M131" s="9" t="str" cm="1">
         <f t="array" ref="M131">PAGE_NAME(B131)</f>
         <v/>
@@ -3515,7 +3518,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="13:14" ht="15.95">
+    <row r="132" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M132" s="9" t="str" cm="1">
         <f t="array" ref="M132">PAGE_NAME(B132)</f>
         <v/>
@@ -3525,7 +3528,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="13:14" ht="15.95">
+    <row r="133" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M133" s="9" t="str" cm="1">
         <f t="array" ref="M133">PAGE_NAME(B133)</f>
         <v/>
@@ -3535,7 +3538,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="13:14" ht="15.95">
+    <row r="134" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M134" s="9" t="str" cm="1">
         <f t="array" ref="M134">PAGE_NAME(B134)</f>
         <v/>
@@ -3545,7 +3548,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="13:14" ht="15.95">
+    <row r="135" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M135" s="9" t="str" cm="1">
         <f t="array" ref="M135">PAGE_NAME(B135)</f>
         <v/>
@@ -3555,7 +3558,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="13:14" ht="15.95">
+    <row r="136" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M136" s="9" t="str" cm="1">
         <f t="array" ref="M136">PAGE_NAME(B136)</f>
         <v/>
@@ -3565,7 +3568,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="13:14" ht="15.95">
+    <row r="137" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M137" s="9" t="str" cm="1">
         <f t="array" ref="M137">PAGE_NAME(B137)</f>
         <v/>
@@ -3575,7 +3578,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="13:14" ht="15.95">
+    <row r="138" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M138" s="9" t="str" cm="1">
         <f t="array" ref="M138">PAGE_NAME(B138)</f>
         <v/>
@@ -3585,7 +3588,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="13:14" ht="15.95">
+    <row r="139" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M139" s="9" t="str" cm="1">
         <f t="array" ref="M139">PAGE_NAME(B139)</f>
         <v/>
@@ -3595,7 +3598,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="13:14" ht="15.95">
+    <row r="140" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M140" s="9" t="str" cm="1">
         <f t="array" ref="M140">PAGE_NAME(B140)</f>
         <v/>
@@ -3605,7 +3608,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="13:14" ht="15.95">
+    <row r="141" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M141" s="9" t="str" cm="1">
         <f t="array" ref="M141">PAGE_NAME(B141)</f>
         <v/>
@@ -3615,7 +3618,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="13:14" ht="15.95">
+    <row r="142" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M142" s="9" t="str" cm="1">
         <f t="array" ref="M142">PAGE_NAME(B142)</f>
         <v/>
@@ -3625,7 +3628,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="13:14" ht="15.95">
+    <row r="143" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M143" s="9" t="str" cm="1">
         <f t="array" ref="M143">PAGE_NAME(B143)</f>
         <v/>
@@ -3635,7 +3638,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="13:14" ht="15.95">
+    <row r="144" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M144" s="9" t="str" cm="1">
         <f t="array" ref="M144">PAGE_NAME(B144)</f>
         <v/>
@@ -3645,7 +3648,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="2:14" ht="15.95">
+    <row r="145" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M145" s="9" t="str" cm="1">
         <f t="array" ref="M145">PAGE_NAME(B145)</f>
         <v/>
@@ -3655,7 +3658,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="2:14" ht="15.95">
+    <row r="146" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M146" s="9" t="str" cm="1">
         <f t="array" ref="M146">PAGE_NAME(B146)</f>
         <v/>
@@ -3665,7 +3668,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="2:14" ht="15.95">
+    <row r="147" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B147" s="11"/>
       <c r="M147" s="9" t="str" cm="1">
         <f t="array" ref="M147">PAGE_NAME(B147)</f>
@@ -3676,7 +3679,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="2:14" ht="15.95">
+    <row r="148" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M148" s="9" t="str" cm="1">
         <f t="array" ref="M148">PAGE_NAME(B148)</f>
         <v/>
@@ -3686,7 +3689,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="2:14" ht="15.95">
+    <row r="149" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M149" s="9" t="str" cm="1">
         <f t="array" ref="M149">PAGE_NAME(B149)</f>
         <v/>
@@ -3696,7 +3699,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="2:14" ht="15.95">
+    <row r="150" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M150" s="9" t="str" cm="1">
         <f t="array" ref="M150">PAGE_NAME(B150)</f>
         <v/>
@@ -3706,7 +3709,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="2:14" ht="15.95">
+    <row r="151" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B151" s="11"/>
       <c r="M151" s="9" t="str" cm="1">
         <f t="array" ref="M151">PAGE_NAME(B151)</f>
@@ -3717,7 +3720,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="2:14" ht="15.95">
+    <row r="152" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M152" s="9" t="str" cm="1">
         <f t="array" ref="M152">PAGE_NAME(B152)</f>
         <v/>
@@ -3727,7 +3730,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="2:14" ht="15.95">
+    <row r="153" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M153" s="9" t="str" cm="1">
         <f t="array" ref="M153">PAGE_NAME(B153)</f>
         <v/>
@@ -3737,7 +3740,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="2:14" ht="15.95">
+    <row r="154" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M154" s="9" t="str" cm="1">
         <f t="array" ref="M154">PAGE_NAME(B154)</f>
         <v/>
@@ -3747,7 +3750,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="2:14" ht="15.95">
+    <row r="155" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M155" s="9" t="str" cm="1">
         <f t="array" ref="M155">PAGE_NAME(B155)</f>
         <v/>
@@ -3757,7 +3760,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="2:14" ht="15.95">
+    <row r="156" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M156" s="9" t="str" cm="1">
         <f t="array" ref="M156">PAGE_NAME(B156)</f>
         <v/>
@@ -3767,7 +3770,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="2:14" ht="15.95">
+    <row r="157" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M157" s="9" t="str" cm="1">
         <f t="array" ref="M157">PAGE_NAME(B157)</f>
         <v/>
@@ -3777,7 +3780,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="2:14" ht="15.95">
+    <row r="158" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M158" s="9" t="str" cm="1">
         <f t="array" ref="M158">PAGE_NAME(B158)</f>
         <v/>
@@ -3787,7 +3790,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="2:14" ht="15.95">
+    <row r="159" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M159" s="9" t="str" cm="1">
         <f t="array" ref="M159">PAGE_NAME(B159)</f>
         <v/>
@@ -3797,7 +3800,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="2:14" ht="15.95">
+    <row r="160" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M160" s="9" t="str" cm="1">
         <f t="array" ref="M160">PAGE_NAME(B160)</f>
         <v/>
@@ -3807,7 +3810,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="2:14" ht="15.95">
+    <row r="161" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M161" s="9" t="str" cm="1">
         <f t="array" ref="M161">PAGE_NAME(B161)</f>
         <v/>
@@ -3817,7 +3820,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="2:14" ht="15.95">
+    <row r="162" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M162" s="9" t="str" cm="1">
         <f t="array" ref="M162">PAGE_NAME(B162)</f>
         <v/>
@@ -3827,7 +3830,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="2:14" ht="15.95">
+    <row r="163" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M163" s="9" t="str" cm="1">
         <f t="array" ref="M163">PAGE_NAME(B163)</f>
         <v/>
@@ -3837,7 +3840,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="2:14" ht="15.95">
+    <row r="164" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M164" s="9" t="str" cm="1">
         <f t="array" ref="M164">PAGE_NAME(B164)</f>
         <v/>
@@ -3847,7 +3850,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="2:14" ht="15.95">
+    <row r="165" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M165" s="9" t="str" cm="1">
         <f t="array" ref="M165">PAGE_NAME(B165)</f>
         <v/>
@@ -3857,7 +3860,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="2:14" ht="15.95">
+    <row r="166" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M166" s="9" t="str" cm="1">
         <f t="array" ref="M166">PAGE_NAME(B166)</f>
         <v/>
@@ -3867,7 +3870,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="2:14" ht="15.95">
+    <row r="167" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M167" s="9" t="str" cm="1">
         <f t="array" ref="M167">PAGE_NAME(B167)</f>
         <v/>
@@ -3877,7 +3880,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="2:14" ht="15.95">
+    <row r="168" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M168" s="9" t="str" cm="1">
         <f t="array" ref="M168">PAGE_NAME(B168)</f>
         <v/>
@@ -3887,7 +3890,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="2:14" ht="15.95">
+    <row r="169" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M169" s="9" t="str" cm="1">
         <f t="array" ref="M169">PAGE_NAME(B169)</f>
         <v/>
@@ -3897,7 +3900,7 @@
         <v/>
       </c>
     </row>
-    <row r="170" spans="2:14" ht="15.95">
+    <row r="170" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M170" s="9" t="str" cm="1">
         <f t="array" ref="M170">PAGE_NAME(B170)</f>
         <v/>
@@ -3907,7 +3910,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="2:14" ht="15.95">
+    <row r="171" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M171" s="9" t="str" cm="1">
         <f t="array" ref="M171">PAGE_NAME(B171)</f>
         <v/>
@@ -3917,7 +3920,7 @@
         <v/>
       </c>
     </row>
-    <row r="172" spans="2:14" ht="15.95">
+    <row r="172" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M172" s="9" t="str" cm="1">
         <f t="array" ref="M172">PAGE_NAME(B172)</f>
         <v/>
@@ -3927,7 +3930,7 @@
         <v/>
       </c>
     </row>
-    <row r="173" spans="2:14" ht="15.95">
+    <row r="173" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M173" s="9" t="str" cm="1">
         <f t="array" ref="M173">PAGE_NAME(B173)</f>
         <v/>
@@ -3937,7 +3940,7 @@
         <v/>
       </c>
     </row>
-    <row r="174" spans="2:14" ht="15.95">
+    <row r="174" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B174"/>
       <c r="M174" s="9" t="str" cm="1">
         <f t="array" ref="M174">PAGE_NAME(B174)</f>
@@ -3948,7 +3951,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" spans="2:14" ht="15.95">
+    <row r="175" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M175" s="9" t="str" cm="1">
         <f t="array" ref="M175">PAGE_NAME(B175)</f>
         <v/>
@@ -3958,7 +3961,7 @@
         <v/>
       </c>
     </row>
-    <row r="176" spans="2:14" ht="15.95">
+    <row r="176" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M176" s="9" t="str" cm="1">
         <f t="array" ref="M176">PAGE_NAME(B176)</f>
         <v/>
@@ -3968,7 +3971,7 @@
         <v/>
       </c>
     </row>
-    <row r="177" spans="13:14" ht="15.95">
+    <row r="177" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M177" s="9" t="str" cm="1">
         <f t="array" ref="M177">PAGE_NAME(B177)</f>
         <v/>
@@ -3978,7 +3981,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="13:14" ht="15.95">
+    <row r="178" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M178" s="9" t="str" cm="1">
         <f t="array" ref="M178">PAGE_NAME(B178)</f>
         <v/>
@@ -3988,7 +3991,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="13:14" ht="15.95">
+    <row r="179" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M179" s="9" t="str" cm="1">
         <f t="array" ref="M179">PAGE_NAME(B179)</f>
         <v/>
@@ -3998,7 +4001,7 @@
         <v/>
       </c>
     </row>
-    <row r="180" spans="13:14" ht="15.95">
+    <row r="180" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M180" s="9" t="str" cm="1">
         <f t="array" ref="M180">PAGE_NAME(B180)</f>
         <v/>
@@ -4008,7 +4011,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="13:14" ht="15.95">
+    <row r="181" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M181" s="9" t="str" cm="1">
         <f t="array" ref="M181">PAGE_NAME(B181)</f>
         <v/>
@@ -4018,7 +4021,7 @@
         <v/>
       </c>
     </row>
-    <row r="182" spans="13:14" ht="15.95">
+    <row r="182" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M182" s="9" t="str" cm="1">
         <f t="array" ref="M182">PAGE_NAME(B182)</f>
         <v/>
@@ -4028,7 +4031,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="13:14" ht="15.95">
+    <row r="183" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M183" s="9" t="str" cm="1">
         <f t="array" ref="M183">PAGE_NAME(B183)</f>
         <v/>
@@ -4038,7 +4041,7 @@
         <v/>
       </c>
     </row>
-    <row r="184" spans="13:14" ht="15.95">
+    <row r="184" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M184" s="9" t="str" cm="1">
         <f t="array" ref="M184">PAGE_NAME(B184)</f>
         <v/>
@@ -4048,7 +4051,7 @@
         <v/>
       </c>
     </row>
-    <row r="185" spans="13:14" ht="15.95">
+    <row r="185" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M185" s="9" t="str" cm="1">
         <f t="array" ref="M185">PAGE_NAME(B185)</f>
         <v/>
@@ -4058,7 +4061,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="13:14" ht="15.95">
+    <row r="186" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M186" s="9" t="str" cm="1">
         <f t="array" ref="M186">PAGE_NAME(B186)</f>
         <v/>
@@ -4068,7 +4071,7 @@
         <v/>
       </c>
     </row>
-    <row r="187" spans="13:14" ht="15.95">
+    <row r="187" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M187" s="9" t="str" cm="1">
         <f t="array" ref="M187">PAGE_NAME(B187)</f>
         <v/>
@@ -4078,7 +4081,7 @@
         <v/>
       </c>
     </row>
-    <row r="188" spans="13:14" ht="15.95">
+    <row r="188" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M188" s="9" t="str" cm="1">
         <f t="array" ref="M188">PAGE_NAME(B188)</f>
         <v/>
@@ -4088,7 +4091,7 @@
         <v/>
       </c>
     </row>
-    <row r="189" spans="13:14" ht="15.95">
+    <row r="189" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M189" s="9" t="str" cm="1">
         <f t="array" ref="M189">PAGE_NAME(B189)</f>
         <v/>
@@ -4098,7 +4101,7 @@
         <v/>
       </c>
     </row>
-    <row r="190" spans="13:14" ht="15.95">
+    <row r="190" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M190" s="9" t="str" cm="1">
         <f t="array" ref="M190">PAGE_NAME(B190)</f>
         <v/>
@@ -4108,7 +4111,7 @@
         <v/>
       </c>
     </row>
-    <row r="191" spans="13:14" ht="15.95">
+    <row r="191" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M191" s="9" t="str" cm="1">
         <f t="array" ref="M191">PAGE_NAME(B191)</f>
         <v/>
@@ -4118,7 +4121,7 @@
         <v/>
       </c>
     </row>
-    <row r="192" spans="13:14" ht="15.95">
+    <row r="192" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M192" s="9" t="str" cm="1">
         <f t="array" ref="M192">PAGE_NAME(B192)</f>
         <v/>
@@ -4128,7 +4131,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="2:14" ht="15.95">
+    <row r="193" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M193" s="9" t="str" cm="1">
         <f t="array" ref="M193">PAGE_NAME(B193)</f>
         <v/>
@@ -4138,7 +4141,7 @@
         <v/>
       </c>
     </row>
-    <row r="194" spans="2:14" ht="15.95">
+    <row r="194" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M194" s="9" t="str" cm="1">
         <f t="array" ref="M194">PAGE_NAME(B194)</f>
         <v/>
@@ -4148,7 +4151,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="2:14" ht="15.95">
+    <row r="195" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M195" s="9" t="str" cm="1">
         <f t="array" ref="M195">PAGE_NAME(B195)</f>
         <v/>
@@ -4158,7 +4161,7 @@
         <v/>
       </c>
     </row>
-    <row r="196" spans="2:14" ht="15.95">
+    <row r="196" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B196" s="11"/>
       <c r="M196" s="9" t="str" cm="1">
         <f t="array" ref="M196">PAGE_NAME(B196)</f>
@@ -4169,7 +4172,7 @@
         <v/>
       </c>
     </row>
-    <row r="197" spans="2:14" ht="15.95">
+    <row r="197" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M197" s="9" t="str" cm="1">
         <f t="array" ref="M197">PAGE_NAME(B197)</f>
         <v/>
@@ -4179,7 +4182,7 @@
         <v/>
       </c>
     </row>
-    <row r="198" spans="2:14" ht="15.95">
+    <row r="198" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M198" s="9" t="str" cm="1">
         <f t="array" ref="M198">PAGE_NAME(B198)</f>
         <v/>
@@ -4189,7 +4192,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="2:14" ht="15.95">
+    <row r="199" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M199" s="9" t="str" cm="1">
         <f t="array" ref="M199">PAGE_NAME(B199)</f>
         <v/>
@@ -4199,7 +4202,7 @@
         <v/>
       </c>
     </row>
-    <row r="200" spans="2:14" ht="15.95">
+    <row r="200" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M200" s="9" t="str" cm="1">
         <f t="array" ref="M200">PAGE_NAME(B200)</f>
         <v/>
@@ -4209,7 +4212,7 @@
         <v/>
       </c>
     </row>
-    <row r="201" spans="2:14" ht="15.95">
+    <row r="201" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M201" s="9" t="str" cm="1">
         <f t="array" ref="M201">PAGE_NAME(B201)</f>
         <v/>
@@ -4219,7 +4222,7 @@
         <v/>
       </c>
     </row>
-    <row r="202" spans="2:14" ht="15.95">
+    <row r="202" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M202" s="9" t="str" cm="1">
         <f t="array" ref="M202">PAGE_NAME(B202)</f>
         <v/>
@@ -4229,7 +4232,7 @@
         <v/>
       </c>
     </row>
-    <row r="203" spans="2:14" ht="15.95">
+    <row r="203" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M203" s="9" t="str" cm="1">
         <f t="array" ref="M203">PAGE_NAME(B203)</f>
         <v/>
@@ -4239,7 +4242,7 @@
         <v/>
       </c>
     </row>
-    <row r="204" spans="2:14" ht="15.95">
+    <row r="204" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M204" s="9" t="str" cm="1">
         <f t="array" ref="M204">PAGE_NAME(B204)</f>
         <v/>
@@ -4249,7 +4252,7 @@
         <v/>
       </c>
     </row>
-    <row r="205" spans="2:14" ht="15.95">
+    <row r="205" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M205" s="9" t="str" cm="1">
         <f t="array" ref="M205">PAGE_NAME(B205)</f>
         <v/>
@@ -4259,7 +4262,7 @@
         <v/>
       </c>
     </row>
-    <row r="206" spans="2:14" ht="15.95">
+    <row r="206" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M206" s="9" t="str" cm="1">
         <f t="array" ref="M206">PAGE_NAME(B206)</f>
         <v/>
@@ -4269,7 +4272,7 @@
         <v/>
       </c>
     </row>
-    <row r="207" spans="2:14" ht="15.95">
+    <row r="207" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M207" s="9" t="str" cm="1">
         <f t="array" ref="M207">PAGE_NAME(B207)</f>
         <v/>
@@ -4279,7 +4282,7 @@
         <v/>
       </c>
     </row>
-    <row r="208" spans="2:14" ht="15.95">
+    <row r="208" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M208" s="9" t="str" cm="1">
         <f t="array" ref="M208">PAGE_NAME(B208)</f>
         <v/>
@@ -4289,7 +4292,7 @@
         <v/>
       </c>
     </row>
-    <row r="209" spans="2:14" ht="15.95">
+    <row r="209" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M209" s="9" t="str" cm="1">
         <f t="array" ref="M209">PAGE_NAME(B209)</f>
         <v/>
@@ -4299,7 +4302,7 @@
         <v/>
       </c>
     </row>
-    <row r="210" spans="2:14" ht="15.95">
+    <row r="210" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M210" s="9" t="str" cm="1">
         <f t="array" ref="M210">PAGE_NAME(B210)</f>
         <v/>
@@ -4309,7 +4312,7 @@
         <v/>
       </c>
     </row>
-    <row r="211" spans="2:14" ht="15.95">
+    <row r="211" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M211" s="9" t="str" cm="1">
         <f t="array" ref="M211">PAGE_NAME(B211)</f>
         <v/>
@@ -4319,7 +4322,7 @@
         <v/>
       </c>
     </row>
-    <row r="212" spans="2:14" ht="15.95">
+    <row r="212" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B212" s="11"/>
       <c r="M212" s="9" t="str" cm="1">
         <f t="array" ref="M212">PAGE_NAME(B212)</f>
@@ -4330,7 +4333,7 @@
         <v/>
       </c>
     </row>
-    <row r="213" spans="2:14" ht="15.95">
+    <row r="213" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B213" s="11"/>
       <c r="M213" s="9" t="str" cm="1">
         <f t="array" ref="M213">PAGE_NAME(B213)</f>
@@ -4341,7 +4344,7 @@
         <v/>
       </c>
     </row>
-    <row r="214" spans="2:14" ht="15.95">
+    <row r="214" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M214" s="9" t="str" cm="1">
         <f t="array" ref="M214">PAGE_NAME(B214)</f>
         <v/>
@@ -4351,7 +4354,7 @@
         <v/>
       </c>
     </row>
-    <row r="215" spans="2:14" ht="15.95">
+    <row r="215" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M215" s="9" t="str" cm="1">
         <f t="array" ref="M215">PAGE_NAME(B215)</f>
         <v/>
@@ -4361,7 +4364,7 @@
         <v/>
       </c>
     </row>
-    <row r="216" spans="2:14" ht="15.95">
+    <row r="216" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M216" s="9" t="str" cm="1">
         <f t="array" ref="M216">PAGE_NAME(B216)</f>
         <v/>
@@ -4371,7 +4374,7 @@
         <v/>
       </c>
     </row>
-    <row r="217" spans="2:14" ht="15.95">
+    <row r="217" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M217" s="9" t="str" cm="1">
         <f t="array" ref="M217">PAGE_NAME(B217)</f>
         <v/>
@@ -4381,7 +4384,7 @@
         <v/>
       </c>
     </row>
-    <row r="218" spans="2:14" ht="15.95">
+    <row r="218" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M218" s="9" t="str" cm="1">
         <f t="array" ref="M218">PAGE_NAME(B218)</f>
         <v/>
@@ -4391,7 +4394,7 @@
         <v/>
       </c>
     </row>
-    <row r="219" spans="2:14" ht="15.95">
+    <row r="219" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M219" s="9" t="str" cm="1">
         <f t="array" ref="M219">PAGE_NAME(B219)</f>
         <v/>
@@ -4401,7 +4404,7 @@
         <v/>
       </c>
     </row>
-    <row r="220" spans="2:14" ht="15.95">
+    <row r="220" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M220" s="9" t="str" cm="1">
         <f t="array" ref="M220">PAGE_NAME(B220)</f>
         <v/>
@@ -4411,7 +4414,7 @@
         <v/>
       </c>
     </row>
-    <row r="221" spans="2:14" ht="15.95">
+    <row r="221" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M221" s="9" t="str" cm="1">
         <f t="array" ref="M221">PAGE_NAME(B221)</f>
         <v/>
@@ -4421,7 +4424,7 @@
         <v/>
       </c>
     </row>
-    <row r="222" spans="2:14" ht="15.95">
+    <row r="222" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M222" s="9" t="str" cm="1">
         <f t="array" ref="M222">PAGE_NAME(B222)</f>
         <v/>
@@ -4431,7 +4434,7 @@
         <v/>
       </c>
     </row>
-    <row r="223" spans="2:14" ht="15.95">
+    <row r="223" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M223" s="9" t="str" cm="1">
         <f t="array" ref="M223">PAGE_NAME(B223)</f>
         <v/>
@@ -4441,7 +4444,7 @@
         <v/>
       </c>
     </row>
-    <row r="224" spans="2:14" ht="15.95">
+    <row r="224" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B224" s="11"/>
       <c r="M224" s="9" t="str" cm="1">
         <f t="array" ref="M224">PAGE_NAME(B224)</f>
@@ -4452,7 +4455,7 @@
         <v/>
       </c>
     </row>
-    <row r="225" spans="2:14" ht="15.95">
+    <row r="225" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B225" s="11"/>
       <c r="M225" s="9" t="str" cm="1">
         <f t="array" ref="M225">PAGE_NAME(B225)</f>
@@ -4463,7 +4466,7 @@
         <v/>
       </c>
     </row>
-    <row r="226" spans="2:14" ht="15.95">
+    <row r="226" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B226" s="11"/>
       <c r="M226" s="9" t="str" cm="1">
         <f t="array" ref="M226">PAGE_NAME(B226)</f>
@@ -4474,7 +4477,7 @@
         <v/>
       </c>
     </row>
-    <row r="227" spans="2:14" ht="15.95">
+    <row r="227" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B227" s="11"/>
       <c r="M227" s="9" t="str" cm="1">
         <f t="array" ref="M227">PAGE_NAME(B227)</f>
@@ -4485,7 +4488,7 @@
         <v/>
       </c>
     </row>
-    <row r="228" spans="2:14" ht="15.95">
+    <row r="228" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B228" s="11"/>
       <c r="M228" s="9" t="str" cm="1">
         <f t="array" ref="M228">PAGE_NAME(B228)</f>
@@ -4496,7 +4499,7 @@
         <v/>
       </c>
     </row>
-    <row r="229" spans="2:14" ht="15.95">
+    <row r="229" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B229" s="11"/>
       <c r="M229" s="9" t="str" cm="1">
         <f t="array" ref="M229">PAGE_NAME(B229)</f>
@@ -4507,7 +4510,7 @@
         <v/>
       </c>
     </row>
-    <row r="230" spans="2:14" ht="15.95">
+    <row r="230" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B230" s="11"/>
       <c r="M230" s="9" t="str" cm="1">
         <f t="array" ref="M230">PAGE_NAME(B230)</f>
@@ -4518,7 +4521,7 @@
         <v/>
       </c>
     </row>
-    <row r="231" spans="2:14" ht="15.95">
+    <row r="231" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B231" s="11"/>
       <c r="M231" s="9" t="str" cm="1">
         <f t="array" ref="M231">PAGE_NAME(B231)</f>
@@ -4529,7 +4532,7 @@
         <v/>
       </c>
     </row>
-    <row r="232" spans="2:14" ht="15.95">
+    <row r="232" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B232" s="11"/>
       <c r="M232" s="9" t="str" cm="1">
         <f t="array" ref="M232">PAGE_NAME(B232)</f>
@@ -4540,7 +4543,7 @@
         <v/>
       </c>
     </row>
-    <row r="233" spans="2:14" ht="15.95">
+    <row r="233" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B233" s="11"/>
       <c r="M233" s="9" t="str" cm="1">
         <f t="array" ref="M233">PAGE_NAME(B233)</f>
@@ -4551,7 +4554,7 @@
         <v/>
       </c>
     </row>
-    <row r="234" spans="2:14" ht="15.95">
+    <row r="234" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B234" s="11"/>
       <c r="M234" s="9" t="str" cm="1">
         <f t="array" ref="M234">PAGE_NAME(B234)</f>
@@ -4562,7 +4565,7 @@
         <v/>
       </c>
     </row>
-    <row r="235" spans="2:14" ht="15.95">
+    <row r="235" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B235" s="11"/>
       <c r="M235" s="9" t="str" cm="1">
         <f t="array" ref="M235">PAGE_NAME(B235)</f>
@@ -4573,7 +4576,7 @@
         <v/>
       </c>
     </row>
-    <row r="236" spans="2:14" ht="15.95">
+    <row r="236" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B236" s="11"/>
       <c r="M236" s="9" t="str" cm="1">
         <f t="array" ref="M236">PAGE_NAME(B236)</f>
@@ -4584,7 +4587,7 @@
         <v/>
       </c>
     </row>
-    <row r="237" spans="2:14" ht="15.95">
+    <row r="237" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B237" s="11"/>
       <c r="M237" s="9" t="str" cm="1">
         <f t="array" ref="M237">PAGE_NAME(B237)</f>
@@ -4595,7 +4598,7 @@
         <v/>
       </c>
     </row>
-    <row r="238" spans="2:14" ht="15.95">
+    <row r="238" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M238" s="9" t="str" cm="1">
         <f t="array" ref="M238">PAGE_NAME(B238)</f>
         <v/>
@@ -4605,7 +4608,7 @@
         <v/>
       </c>
     </row>
-    <row r="239" spans="2:14" ht="15.95">
+    <row r="239" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M239" s="9" t="str" cm="1">
         <f t="array" ref="M239">PAGE_NAME(B239)</f>
         <v/>
@@ -4615,7 +4618,7 @@
         <v/>
       </c>
     </row>
-    <row r="240" spans="2:14" ht="15.95">
+    <row r="240" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M240" s="9" t="str" cm="1">
         <f t="array" ref="M240">PAGE_NAME(B240)</f>
         <v/>
@@ -4625,7 +4628,7 @@
         <v/>
       </c>
     </row>
-    <row r="241" spans="13:14" ht="15.95">
+    <row r="241" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M241" s="9" t="str" cm="1">
         <f t="array" ref="M241">PAGE_NAME(B241)</f>
         <v/>
@@ -4635,7 +4638,7 @@
         <v/>
       </c>
     </row>
-    <row r="242" spans="13:14" ht="15.95">
+    <row r="242" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M242" s="9" t="str" cm="1">
         <f t="array" ref="M242">PAGE_NAME(B242)</f>
         <v/>
@@ -4645,7 +4648,7 @@
         <v/>
       </c>
     </row>
-    <row r="243" spans="13:14" ht="15.95">
+    <row r="243" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M243" s="9" t="str" cm="1">
         <f t="array" ref="M243">PAGE_NAME(B243)</f>
         <v/>
@@ -4655,7 +4658,7 @@
         <v/>
       </c>
     </row>
-    <row r="244" spans="13:14" ht="15.95">
+    <row r="244" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M244" s="9" t="str" cm="1">
         <f t="array" ref="M244">PAGE_NAME(B244)</f>
         <v/>
@@ -4665,7 +4668,7 @@
         <v/>
       </c>
     </row>
-    <row r="245" spans="13:14" ht="15.95">
+    <row r="245" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M245" s="9" t="str" cm="1">
         <f t="array" ref="M245">PAGE_NAME(B245)</f>
         <v/>
@@ -4675,7 +4678,7 @@
         <v/>
       </c>
     </row>
-    <row r="246" spans="13:14" ht="15.95">
+    <row r="246" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M246" s="9" t="str" cm="1">
         <f t="array" ref="M246">PAGE_NAME(B246)</f>
         <v/>
@@ -4685,7 +4688,7 @@
         <v/>
       </c>
     </row>
-    <row r="247" spans="13:14" ht="15.95">
+    <row r="247" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M247" s="9" t="str" cm="1">
         <f t="array" ref="M247">PAGE_NAME(B247)</f>
         <v/>
@@ -4695,7 +4698,7 @@
         <v/>
       </c>
     </row>
-    <row r="248" spans="13:14" ht="15.95">
+    <row r="248" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M248" s="9" t="str" cm="1">
         <f t="array" ref="M248">PAGE_NAME(B248)</f>
         <v/>
@@ -4705,7 +4708,7 @@
         <v/>
       </c>
     </row>
-    <row r="249" spans="13:14" ht="15.95">
+    <row r="249" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M249" s="9" t="str" cm="1">
         <f t="array" ref="M249">PAGE_NAME(B249)</f>
         <v/>
@@ -4715,7 +4718,7 @@
         <v/>
       </c>
     </row>
-    <row r="250" spans="13:14" ht="15.95">
+    <row r="250" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M250" s="9" t="str" cm="1">
         <f t="array" ref="M250">PAGE_NAME(B250)</f>
         <v/>
@@ -4725,7 +4728,7 @@
         <v/>
       </c>
     </row>
-    <row r="251" spans="13:14" ht="15.95">
+    <row r="251" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M251" s="9" t="str" cm="1">
         <f t="array" ref="M251">PAGE_NAME(B251)</f>
         <v/>
@@ -4735,7 +4738,7 @@
         <v/>
       </c>
     </row>
-    <row r="252" spans="13:14" ht="15.95">
+    <row r="252" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M252" s="9" t="str" cm="1">
         <f t="array" ref="M252">PAGE_NAME(B252)</f>
         <v/>
@@ -4745,7 +4748,7 @@
         <v/>
       </c>
     </row>
-    <row r="253" spans="13:14" ht="15.95">
+    <row r="253" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M253" s="9" t="str" cm="1">
         <f t="array" ref="M253">PAGE_NAME(B253)</f>
         <v/>
@@ -4755,7 +4758,7 @@
         <v/>
       </c>
     </row>
-    <row r="254" spans="13:14" ht="15.95">
+    <row r="254" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M254" s="9" t="str" cm="1">
         <f t="array" ref="M254">PAGE_NAME(B254)</f>
         <v/>
@@ -4765,7 +4768,7 @@
         <v/>
       </c>
     </row>
-    <row r="255" spans="13:14" ht="15.95">
+    <row r="255" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M255" s="9" t="str" cm="1">
         <f t="array" ref="M255">PAGE_NAME(B255)</f>
         <v/>
@@ -4775,7 +4778,7 @@
         <v/>
       </c>
     </row>
-    <row r="256" spans="13:14" ht="15.95">
+    <row r="256" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M256" s="9" t="str" cm="1">
         <f t="array" ref="M256">PAGE_NAME(B256)</f>
         <v/>
@@ -4785,7 +4788,7 @@
         <v/>
       </c>
     </row>
-    <row r="257" spans="2:14" ht="15.95">
+    <row r="257" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M257" s="9" t="str" cm="1">
         <f t="array" ref="M257">PAGE_NAME(B257)</f>
         <v/>
@@ -4795,7 +4798,7 @@
         <v/>
       </c>
     </row>
-    <row r="258" spans="2:14" ht="15.95">
+    <row r="258" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="B258" s="11"/>
       <c r="M258" s="9" t="str" cm="1">
         <f t="array" ref="M258">PAGE_NAME(B258)</f>
@@ -4806,7 +4809,7 @@
         <v/>
       </c>
     </row>
-    <row r="259" spans="2:14" ht="15.95">
+    <row r="259" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M259" s="9" t="str" cm="1">
         <f t="array" ref="M259">PAGE_NAME(B259)</f>
         <v/>
@@ -4816,7 +4819,7 @@
         <v/>
       </c>
     </row>
-    <row r="260" spans="2:14" ht="15.95">
+    <row r="260" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M260" s="9" t="str" cm="1">
         <f t="array" ref="M260">PAGE_NAME(B260)</f>
         <v/>
@@ -4826,7 +4829,7 @@
         <v/>
       </c>
     </row>
-    <row r="261" spans="2:14" ht="15.95">
+    <row r="261" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M261" s="9" t="str" cm="1">
         <f t="array" ref="M261">PAGE_NAME(B261)</f>
         <v/>
@@ -4836,7 +4839,7 @@
         <v/>
       </c>
     </row>
-    <row r="262" spans="2:14" ht="15.95">
+    <row r="262" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M262" s="9" t="str" cm="1">
         <f t="array" ref="M262">PAGE_NAME(B262)</f>
         <v/>
@@ -4846,7 +4849,7 @@
         <v/>
       </c>
     </row>
-    <row r="263" spans="2:14" ht="15.95">
+    <row r="263" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M263" s="9" t="str" cm="1">
         <f t="array" ref="M263">PAGE_NAME(B263)</f>
         <v/>
@@ -4856,7 +4859,7 @@
         <v/>
       </c>
     </row>
-    <row r="264" spans="2:14" ht="15.95">
+    <row r="264" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M264" s="9" t="str" cm="1">
         <f t="array" ref="M264">PAGE_NAME(B264)</f>
         <v/>
@@ -4866,7 +4869,7 @@
         <v/>
       </c>
     </row>
-    <row r="265" spans="2:14" ht="15.95">
+    <row r="265" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M265" s="9" t="str" cm="1">
         <f t="array" ref="M265">PAGE_NAME(B265)</f>
         <v/>
@@ -4876,7 +4879,7 @@
         <v/>
       </c>
     </row>
-    <row r="266" spans="2:14" ht="15.95">
+    <row r="266" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M266" s="9" t="str" cm="1">
         <f t="array" ref="M266">PAGE_NAME(B266)</f>
         <v/>
@@ -4886,7 +4889,7 @@
         <v/>
       </c>
     </row>
-    <row r="267" spans="2:14" ht="15.95">
+    <row r="267" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M267" s="9" t="str" cm="1">
         <f t="array" ref="M267">PAGE_NAME(B267)</f>
         <v/>
@@ -4896,7 +4899,7 @@
         <v/>
       </c>
     </row>
-    <row r="268" spans="2:14" ht="15.95">
+    <row r="268" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M268" s="9" t="str" cm="1">
         <f t="array" ref="M268">PAGE_NAME(B268)</f>
         <v/>
@@ -4906,7 +4909,7 @@
         <v/>
       </c>
     </row>
-    <row r="269" spans="2:14" ht="15.95">
+    <row r="269" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M269" s="9" t="str" cm="1">
         <f t="array" ref="M269">PAGE_NAME(B269)</f>
         <v/>
@@ -4916,7 +4919,7 @@
         <v/>
       </c>
     </row>
-    <row r="270" spans="2:14" ht="15.95">
+    <row r="270" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M270" s="9" t="str" cm="1">
         <f t="array" ref="M270">PAGE_NAME(B270)</f>
         <v/>
@@ -4926,7 +4929,7 @@
         <v/>
       </c>
     </row>
-    <row r="271" spans="2:14" ht="15.95">
+    <row r="271" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M271" s="9" t="str" cm="1">
         <f t="array" ref="M271">PAGE_NAME(B271)</f>
         <v/>
@@ -4936,7 +4939,7 @@
         <v/>
       </c>
     </row>
-    <row r="272" spans="2:14" ht="15.95">
+    <row r="272" spans="2:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M272" s="9" t="str" cm="1">
         <f t="array" ref="M272">PAGE_NAME(B272)</f>
         <v/>
@@ -4946,7 +4949,7 @@
         <v/>
       </c>
     </row>
-    <row r="273" spans="13:14" ht="15.95">
+    <row r="273" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M273" s="9" t="str" cm="1">
         <f t="array" ref="M273">PAGE_NAME(B273)</f>
         <v/>
@@ -4956,7 +4959,7 @@
         <v/>
       </c>
     </row>
-    <row r="274" spans="13:14" ht="15.95">
+    <row r="274" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M274" s="9" t="str" cm="1">
         <f t="array" ref="M274">PAGE_NAME(B274)</f>
         <v/>
@@ -4966,7 +4969,7 @@
         <v/>
       </c>
     </row>
-    <row r="275" spans="13:14" ht="15.95">
+    <row r="275" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M275" s="9" t="str" cm="1">
         <f t="array" ref="M275">PAGE_NAME(B275)</f>
         <v/>
@@ -4976,7 +4979,7 @@
         <v/>
       </c>
     </row>
-    <row r="276" spans="13:14" ht="15.95">
+    <row r="276" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M276" s="9" t="str" cm="1">
         <f t="array" ref="M276">PAGE_NAME(B276)</f>
         <v/>
@@ -4986,7 +4989,7 @@
         <v/>
       </c>
     </row>
-    <row r="277" spans="13:14" ht="15.95">
+    <row r="277" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M277" s="9" t="str" cm="1">
         <f t="array" ref="M277">PAGE_NAME(B277)</f>
         <v/>
@@ -4996,7 +4999,7 @@
         <v/>
       </c>
     </row>
-    <row r="278" spans="13:14" ht="15.95">
+    <row r="278" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M278" s="9" t="str" cm="1">
         <f t="array" ref="M278">PAGE_NAME(B278)</f>
         <v/>
@@ -5006,7 +5009,7 @@
         <v/>
       </c>
     </row>
-    <row r="279" spans="13:14" ht="15.95">
+    <row r="279" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M279" s="9" t="str" cm="1">
         <f t="array" ref="M279">PAGE_NAME(B279)</f>
         <v/>
@@ -5016,7 +5019,7 @@
         <v/>
       </c>
     </row>
-    <row r="280" spans="13:14" ht="15.95">
+    <row r="280" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M280" s="9" t="str" cm="1">
         <f t="array" ref="M280">PAGE_NAME(B280)</f>
         <v/>
@@ -5026,7 +5029,7 @@
         <v/>
       </c>
     </row>
-    <row r="281" spans="13:14" ht="15.95">
+    <row r="281" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M281" s="9" t="str" cm="1">
         <f t="array" ref="M281">PAGE_NAME(B281)</f>
         <v/>
@@ -5036,7 +5039,7 @@
         <v/>
       </c>
     </row>
-    <row r="282" spans="13:14" ht="15.95">
+    <row r="282" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M282" s="9" t="str" cm="1">
         <f t="array" ref="M282">PAGE_NAME(B282)</f>
         <v/>
@@ -5046,7 +5049,7 @@
         <v/>
       </c>
     </row>
-    <row r="283" spans="13:14" ht="15.95">
+    <row r="283" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M283" s="9" t="str" cm="1">
         <f t="array" ref="M283">PAGE_NAME(B283)</f>
         <v/>
@@ -5056,7 +5059,7 @@
         <v/>
       </c>
     </row>
-    <row r="284" spans="13:14" ht="15.95">
+    <row r="284" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M284" s="9" t="str" cm="1">
         <f t="array" ref="M284">PAGE_NAME(B284)</f>
         <v/>
@@ -5066,7 +5069,7 @@
         <v/>
       </c>
     </row>
-    <row r="285" spans="13:14" ht="15.95">
+    <row r="285" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M285" s="9" t="str" cm="1">
         <f t="array" ref="M285">PAGE_NAME(B285)</f>
         <v/>
@@ -5076,7 +5079,7 @@
         <v/>
       </c>
     </row>
-    <row r="286" spans="13:14" ht="15.95">
+    <row r="286" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M286" s="9" t="str" cm="1">
         <f t="array" ref="M286">PAGE_NAME(B286)</f>
         <v/>
@@ -5086,7 +5089,7 @@
         <v/>
       </c>
     </row>
-    <row r="287" spans="13:14" ht="15.95">
+    <row r="287" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M287" s="9" t="str" cm="1">
         <f t="array" ref="M287">PAGE_NAME(B287)</f>
         <v/>
@@ -5096,7 +5099,7 @@
         <v/>
       </c>
     </row>
-    <row r="288" spans="13:14" ht="15.95">
+    <row r="288" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M288" s="9" t="str" cm="1">
         <f t="array" ref="M288">PAGE_NAME(B288)</f>
         <v/>
@@ -5106,7 +5109,7 @@
         <v/>
       </c>
     </row>
-    <row r="289" spans="13:14" ht="15.95">
+    <row r="289" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M289" s="9" t="str" cm="1">
         <f t="array" ref="M289">PAGE_NAME(B289)</f>
         <v/>
@@ -5116,7 +5119,7 @@
         <v/>
       </c>
     </row>
-    <row r="290" spans="13:14" ht="15.95">
+    <row r="290" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M290" s="9" t="str" cm="1">
         <f t="array" ref="M290">PAGE_NAME(B290)</f>
         <v/>
@@ -5126,7 +5129,7 @@
         <v/>
       </c>
     </row>
-    <row r="291" spans="13:14" ht="15.95">
+    <row r="291" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M291" s="9" t="str" cm="1">
         <f t="array" ref="M291">PAGE_NAME(B291)</f>
         <v/>
@@ -5136,7 +5139,7 @@
         <v/>
       </c>
     </row>
-    <row r="292" spans="13:14" ht="15.95">
+    <row r="292" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M292" s="9" t="str" cm="1">
         <f t="array" ref="M292">PAGE_NAME(B292)</f>
         <v/>
@@ -5146,7 +5149,7 @@
         <v/>
       </c>
     </row>
-    <row r="293" spans="13:14" ht="15.95">
+    <row r="293" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M293" s="9" t="str" cm="1">
         <f t="array" ref="M293">PAGE_NAME(B293)</f>
         <v/>
@@ -5156,7 +5159,7 @@
         <v/>
       </c>
     </row>
-    <row r="294" spans="13:14" ht="15.95">
+    <row r="294" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M294" s="9" t="str" cm="1">
         <f t="array" ref="M294">PAGE_NAME(B294)</f>
         <v/>
@@ -5166,7 +5169,7 @@
         <v/>
       </c>
     </row>
-    <row r="295" spans="13:14" ht="15.95">
+    <row r="295" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M295" s="9" t="str" cm="1">
         <f t="array" ref="M295">PAGE_NAME(B295)</f>
         <v/>
@@ -5176,7 +5179,7 @@
         <v/>
       </c>
     </row>
-    <row r="296" spans="13:14" ht="15.95">
+    <row r="296" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M296" s="9" t="str" cm="1">
         <f t="array" ref="M296">PAGE_NAME(B296)</f>
         <v/>
@@ -5186,7 +5189,7 @@
         <v/>
       </c>
     </row>
-    <row r="297" spans="13:14" ht="15.95">
+    <row r="297" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M297" s="9" t="str" cm="1">
         <f t="array" ref="M297">PAGE_NAME(B297)</f>
         <v/>
@@ -5196,7 +5199,7 @@
         <v/>
       </c>
     </row>
-    <row r="298" spans="13:14" ht="15.95">
+    <row r="298" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M298" s="9" t="str" cm="1">
         <f t="array" ref="M298">PAGE_NAME(B298)</f>
         <v/>
@@ -5206,7 +5209,7 @@
         <v/>
       </c>
     </row>
-    <row r="299" spans="13:14" ht="15.95">
+    <row r="299" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M299" s="9" t="str" cm="1">
         <f t="array" ref="M299">PAGE_NAME(B299)</f>
         <v/>
@@ -5216,7 +5219,7 @@
         <v/>
       </c>
     </row>
-    <row r="300" spans="13:14" ht="15.95">
+    <row r="300" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M300" s="9" t="str" cm="1">
         <f t="array" ref="M300">PAGE_NAME(B300)</f>
         <v/>
@@ -5226,7 +5229,7 @@
         <v/>
       </c>
     </row>
-    <row r="301" spans="13:14" ht="15.95">
+    <row r="301" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M301" s="9" t="str" cm="1">
         <f t="array" ref="M301">PAGE_NAME(B301)</f>
         <v/>
@@ -5236,7 +5239,7 @@
         <v/>
       </c>
     </row>
-    <row r="302" spans="13:14" ht="15.95">
+    <row r="302" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M302" s="9" t="str" cm="1">
         <f t="array" ref="M302">PAGE_NAME(B302)</f>
         <v/>
@@ -5246,7 +5249,7 @@
         <v/>
       </c>
     </row>
-    <row r="303" spans="13:14" ht="15.95">
+    <row r="303" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M303" s="9" t="str" cm="1">
         <f t="array" ref="M303">PAGE_NAME(B303)</f>
         <v/>
@@ -5256,7 +5259,7 @@
         <v/>
       </c>
     </row>
-    <row r="304" spans="13:14" ht="15.95">
+    <row r="304" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M304" s="9" t="str" cm="1">
         <f t="array" ref="M304">PAGE_NAME(B304)</f>
         <v/>
@@ -5266,7 +5269,7 @@
         <v/>
       </c>
     </row>
-    <row r="305" spans="13:14" ht="15.95">
+    <row r="305" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M305" s="9" t="str" cm="1">
         <f t="array" ref="M305">PAGE_NAME(B305)</f>
         <v/>
@@ -5276,7 +5279,7 @@
         <v/>
       </c>
     </row>
-    <row r="306" spans="13:14" ht="15.95">
+    <row r="306" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M306" s="9" t="str" cm="1">
         <f t="array" ref="M306">PAGE_NAME(B306)</f>
         <v/>
@@ -5286,7 +5289,7 @@
         <v/>
       </c>
     </row>
-    <row r="307" spans="13:14" ht="15.95">
+    <row r="307" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M307" s="9" t="str" cm="1">
         <f t="array" ref="M307">PAGE_NAME(B307)</f>
         <v/>
@@ -5296,7 +5299,7 @@
         <v/>
       </c>
     </row>
-    <row r="308" spans="13:14" ht="15.95">
+    <row r="308" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M308" s="9" t="str" cm="1">
         <f t="array" ref="M308">PAGE_NAME(B308)</f>
         <v/>
@@ -5306,7 +5309,7 @@
         <v/>
       </c>
     </row>
-    <row r="309" spans="13:14" ht="15.95">
+    <row r="309" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M309" s="9" t="str" cm="1">
         <f t="array" ref="M309">PAGE_NAME(B309)</f>
         <v/>
@@ -5316,7 +5319,7 @@
         <v/>
       </c>
     </row>
-    <row r="310" spans="13:14" ht="15.95">
+    <row r="310" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M310" s="9" t="str" cm="1">
         <f t="array" ref="M310">PAGE_NAME(B310)</f>
         <v/>
@@ -5326,7 +5329,7 @@
         <v/>
       </c>
     </row>
-    <row r="311" spans="13:14" ht="15.95">
+    <row r="311" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M311" s="9" t="str" cm="1">
         <f t="array" ref="M311">PAGE_NAME(B311)</f>
         <v/>
@@ -5336,7 +5339,7 @@
         <v/>
       </c>
     </row>
-    <row r="312" spans="13:14" ht="15.95">
+    <row r="312" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M312" s="9" t="str" cm="1">
         <f t="array" ref="M312">PAGE_NAME(B312)</f>
         <v/>
@@ -5346,7 +5349,7 @@
         <v/>
       </c>
     </row>
-    <row r="313" spans="13:14" ht="15.95">
+    <row r="313" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M313" s="9" t="str" cm="1">
         <f t="array" ref="M313">PAGE_NAME(B313)</f>
         <v/>
@@ -5356,7 +5359,7 @@
         <v/>
       </c>
     </row>
-    <row r="314" spans="13:14" ht="15.95">
+    <row r="314" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M314" s="9" t="str" cm="1">
         <f t="array" ref="M314">PAGE_NAME(B314)</f>
         <v/>
@@ -5366,7 +5369,7 @@
         <v/>
       </c>
     </row>
-    <row r="315" spans="13:14" ht="15.95">
+    <row r="315" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M315" s="9" t="str" cm="1">
         <f t="array" ref="M315">PAGE_NAME(B315)</f>
         <v/>
@@ -5376,7 +5379,7 @@
         <v/>
       </c>
     </row>
-    <row r="316" spans="13:14" ht="15.95">
+    <row r="316" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M316" s="9" t="str" cm="1">
         <f t="array" ref="M316">PAGE_NAME(B316)</f>
         <v/>
@@ -5386,7 +5389,7 @@
         <v/>
       </c>
     </row>
-    <row r="317" spans="13:14" ht="15.95">
+    <row r="317" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M317" s="9" t="str" cm="1">
         <f t="array" ref="M317">PAGE_NAME(B317)</f>
         <v/>
@@ -5396,7 +5399,7 @@
         <v/>
       </c>
     </row>
-    <row r="318" spans="13:14" ht="15.95">
+    <row r="318" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M318" s="9" t="str" cm="1">
         <f t="array" ref="M318">PAGE_NAME(B318)</f>
         <v/>
@@ -5406,7 +5409,7 @@
         <v/>
       </c>
     </row>
-    <row r="319" spans="13:14" ht="15.95">
+    <row r="319" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M319" s="9" t="str" cm="1">
         <f t="array" ref="M319">PAGE_NAME(B319)</f>
         <v/>
@@ -5416,7 +5419,7 @@
         <v/>
       </c>
     </row>
-    <row r="320" spans="13:14" ht="15.95">
+    <row r="320" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M320" s="9" t="str" cm="1">
         <f t="array" ref="M320">PAGE_NAME(B320)</f>
         <v/>
@@ -5426,7 +5429,7 @@
         <v/>
       </c>
     </row>
-    <row r="321" spans="13:14" ht="15.95">
+    <row r="321" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M321" s="9" t="str" cm="1">
         <f t="array" ref="M321">PAGE_NAME(B321)</f>
         <v/>
@@ -5436,7 +5439,7 @@
         <v/>
       </c>
     </row>
-    <row r="322" spans="13:14" ht="15.95">
+    <row r="322" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M322" s="9" t="str" cm="1">
         <f t="array" ref="M322">PAGE_NAME(B322)</f>
         <v/>
@@ -5446,7 +5449,7 @@
         <v/>
       </c>
     </row>
-    <row r="323" spans="13:14" ht="15.95">
+    <row r="323" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M323" s="9" t="str" cm="1">
         <f t="array" ref="M323">PAGE_NAME(B323)</f>
         <v/>
@@ -5456,7 +5459,7 @@
         <v/>
       </c>
     </row>
-    <row r="324" spans="13:14" ht="15.95">
+    <row r="324" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M324" s="9" t="str" cm="1">
         <f t="array" ref="M324">PAGE_NAME(B324)</f>
         <v/>
@@ -5466,7 +5469,7 @@
         <v/>
       </c>
     </row>
-    <row r="325" spans="13:14" ht="15.95">
+    <row r="325" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M325" s="9" t="str" cm="1">
         <f t="array" ref="M325">PAGE_NAME(B325)</f>
         <v/>
@@ -5476,7 +5479,7 @@
         <v/>
       </c>
     </row>
-    <row r="326" spans="13:14" ht="15.95">
+    <row r="326" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M326" s="9" t="str" cm="1">
         <f t="array" ref="M326">PAGE_NAME(B326)</f>
         <v/>
@@ -5486,7 +5489,7 @@
         <v/>
       </c>
     </row>
-    <row r="327" spans="13:14" ht="15.95">
+    <row r="327" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M327" s="9" t="str" cm="1">
         <f t="array" ref="M327">PAGE_NAME(B327)</f>
         <v/>
@@ -5496,7 +5499,7 @@
         <v/>
       </c>
     </row>
-    <row r="328" spans="13:14" ht="15.95">
+    <row r="328" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M328" s="9" t="str" cm="1">
         <f t="array" ref="M328">PAGE_NAME(B328)</f>
         <v/>
@@ -5506,7 +5509,7 @@
         <v/>
       </c>
     </row>
-    <row r="329" spans="13:14" ht="15.95">
+    <row r="329" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M329" s="9" t="str" cm="1">
         <f t="array" ref="M329">PAGE_NAME(B329)</f>
         <v/>
@@ -5516,7 +5519,7 @@
         <v/>
       </c>
     </row>
-    <row r="330" spans="13:14" ht="15.95">
+    <row r="330" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M330" s="9" t="str" cm="1">
         <f t="array" ref="M330">PAGE_NAME(B330)</f>
         <v/>
@@ -5526,7 +5529,7 @@
         <v/>
       </c>
     </row>
-    <row r="331" spans="13:14" ht="15.95">
+    <row r="331" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M331" s="9" t="str" cm="1">
         <f t="array" ref="M331">PAGE_NAME(B331)</f>
         <v/>
@@ -5536,7 +5539,7 @@
         <v/>
       </c>
     </row>
-    <row r="332" spans="13:14" ht="15.95">
+    <row r="332" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M332" s="9" t="str" cm="1">
         <f t="array" ref="M332">PAGE_NAME(B332)</f>
         <v/>
@@ -5546,7 +5549,7 @@
         <v/>
       </c>
     </row>
-    <row r="333" spans="13:14" ht="15.95">
+    <row r="333" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M333" s="9" t="str" cm="1">
         <f t="array" ref="M333">PAGE_NAME(B333)</f>
         <v/>
@@ -5556,7 +5559,7 @@
         <v/>
       </c>
     </row>
-    <row r="334" spans="13:14" ht="15.95">
+    <row r="334" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M334" s="9" t="str" cm="1">
         <f t="array" ref="M334">PAGE_NAME(B334)</f>
         <v/>
@@ -5566,7 +5569,7 @@
         <v/>
       </c>
     </row>
-    <row r="335" spans="13:14" ht="15.95">
+    <row r="335" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M335" s="9" t="str" cm="1">
         <f t="array" ref="M335">PAGE_NAME(B335)</f>
         <v/>
@@ -5576,7 +5579,7 @@
         <v/>
       </c>
     </row>
-    <row r="336" spans="13:14" ht="15.95">
+    <row r="336" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M336" s="9" t="str" cm="1">
         <f t="array" ref="M336">PAGE_NAME(B336)</f>
         <v/>
@@ -5586,7 +5589,7 @@
         <v/>
       </c>
     </row>
-    <row r="337" spans="13:14" ht="15.95">
+    <row r="337" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M337" s="9" t="str" cm="1">
         <f t="array" ref="M337">PAGE_NAME(B337)</f>
         <v/>
@@ -5596,7 +5599,7 @@
         <v/>
       </c>
     </row>
-    <row r="338" spans="13:14" ht="15.95">
+    <row r="338" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M338" s="9" t="str" cm="1">
         <f t="array" ref="M338">PAGE_NAME(B338)</f>
         <v/>
@@ -5606,7 +5609,7 @@
         <v/>
       </c>
     </row>
-    <row r="339" spans="13:14" ht="15.95">
+    <row r="339" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M339" s="9" t="str" cm="1">
         <f t="array" ref="M339">PAGE_NAME(B339)</f>
         <v/>
@@ -5616,7 +5619,7 @@
         <v/>
       </c>
     </row>
-    <row r="340" spans="13:14" ht="15.95">
+    <row r="340" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M340" s="9" t="str" cm="1">
         <f t="array" ref="M340">PAGE_NAME(B340)</f>
         <v/>
@@ -5626,7 +5629,7 @@
         <v/>
       </c>
     </row>
-    <row r="341" spans="13:14" ht="15.95">
+    <row r="341" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M341" s="9" t="str" cm="1">
         <f t="array" ref="M341">PAGE_NAME(B341)</f>
         <v/>
@@ -5636,7 +5639,7 @@
         <v/>
       </c>
     </row>
-    <row r="342" spans="13:14" ht="15.95">
+    <row r="342" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M342" s="9" t="str" cm="1">
         <f t="array" ref="M342">PAGE_NAME(B342)</f>
         <v/>
@@ -5646,7 +5649,7 @@
         <v/>
       </c>
     </row>
-    <row r="343" spans="13:14" ht="15.95">
+    <row r="343" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M343" s="9" t="str" cm="1">
         <f t="array" ref="M343">PAGE_NAME(B343)</f>
         <v/>
@@ -5656,7 +5659,7 @@
         <v/>
       </c>
     </row>
-    <row r="344" spans="13:14" ht="15.95">
+    <row r="344" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M344" s="9" t="str" cm="1">
         <f t="array" ref="M344">PAGE_NAME(B344)</f>
         <v/>
@@ -5666,7 +5669,7 @@
         <v/>
       </c>
     </row>
-    <row r="345" spans="13:14" ht="15.95">
+    <row r="345" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M345" s="9" t="str" cm="1">
         <f t="array" ref="M345">PAGE_NAME(B345)</f>
         <v/>
@@ -5676,7 +5679,7 @@
         <v/>
       </c>
     </row>
-    <row r="346" spans="13:14" ht="15.95">
+    <row r="346" spans="13:14" ht="16" x14ac:dyDescent="0.2">
       <c r="M346" s="9" t="str" cm="1">
         <f t="array" ref="M346">PAGE_NAME(B346)</f>
         <v/>
@@ -5688,15 +5691,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{13A1A56B-038A-43A9-B92C-DA261D9E629C}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{65FA32E5-A89D-4CA0-B1E1-01AB95B97F01}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{82548974-4169-476D-A33A-D8AA97B9D7F0}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{FEB47017-D5EA-402E-9A45-ED12D6969DD0}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{AF8D38BC-C7D7-4026-A283-7ACD654CE59A}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{6CEA468A-2770-42F2-8A8B-A11DBB84D887}"/>
-    <hyperlink ref="B8" r:id="rId7" xr:uid="{43FEDD78-80F9-4CD3-A668-88CC83C591CF}"/>
-    <hyperlink ref="B9" r:id="rId8" xr:uid="{2699103D-3D39-4ECE-A1B3-19D33FE3458A}"/>
-    <hyperlink ref="B10" r:id="rId9" xr:uid="{3C6E4BC8-E64E-46BA-8C03-3B55352AD14F}"/>
+    <hyperlink ref="B3" r:id="rId1" location="p-170.315(g)(33)(i)" xr:uid="{65FA32E5-A89D-4CA0-B1E1-01AB95B97F01}"/>
+    <hyperlink ref="B4" r:id="rId2" location="p-170.315(g)(33)(i)(A)" xr:uid="{82548974-4169-476D-A33A-D8AA97B9D7F0}"/>
+    <hyperlink ref="B5" r:id="rId3" location="p-170.315(g)(33)(i)(B)" xr:uid="{FEB47017-D5EA-402E-9A45-ED12D6969DD0}"/>
+    <hyperlink ref="B6" r:id="rId4" location="p-170.315(g)(33)(i)©" xr:uid="{AF8D38BC-C7D7-4026-A283-7ACD654CE59A}"/>
+    <hyperlink ref="B7" r:id="rId5" location="p-170.315(g)(33)(i)(C)(1)" xr:uid="{6CEA468A-2770-42F2-8A8B-A11DBB84D887}"/>
+    <hyperlink ref="B8" r:id="rId6" location="p-170.315(g)(33)(i)(C)(2)" xr:uid="{43FEDD78-80F9-4CD3-A668-88CC83C591CF}"/>
+    <hyperlink ref="B9" r:id="rId7" location="p-170.315(g)(33)(i)(C)(3)" xr:uid="{2699103D-3D39-4ECE-A1B3-19D33FE3458A}"/>
+    <hyperlink ref="B10" r:id="rId8" location="p-170.315(g)(33)(ii)" xr:uid="{3C6E4BC8-E64E-46BA-8C03-3B55352AD14F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -5729,84 +5731,84 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C323F474-BE25-4449-9222-E1A46A1843B5}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="56.5" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="408.95" customHeight="1">
+    <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="41" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="41"/>
     </row>
-    <row r="2" spans="1:2" ht="81.95" customHeight="1">
+    <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="41"/>
       <c r="B2" s="41"/>
     </row>
-    <row r="3" spans="1:2" ht="15.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="18" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="B4" s="33" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="18" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="18" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="18" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="18" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -5823,41 +5825,41 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C49B4E29-A057-6044-8543-9F9FC3A9F2DF}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="3" width="14.625" customWidth="1"/>
+    <col min="2" max="3" width="14.6640625" customWidth="1"/>
     <col min="4" max="4" width="29.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0.1</v>
       </c>
       <c r="B2" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="C2" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="D2" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -5868,23 +5870,23 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AB89888-9517-1640-A922-49BDADD5811C}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="B1" t="s">
         <v>42</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="D1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>86</v>
       </c>
@@ -5892,47 +5894,47 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="D2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="B3" t="b">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="C4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -5941,23 +5943,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Notes xmlns="5c50ed2d-852b-4196-83c6-52aa9500028d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001741AA2D27F8C248A1151A0995DC29E6" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f19764ae00be838914eeb4c0c1ffa724">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5c50ed2d-852b-4196-83c6-52aa9500028d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="115b5e86e2dc776b9e9357163dc7f5dc" ns2:_="">
     <xsd:import namespace="5c50ed2d-852b-4196-83c6-52aa9500028d"/>
@@ -6127,14 +6112,55 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Notes xmlns="5c50ed2d-852b-4196-83c6-52aa9500028d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93316912-AE26-426F-A937-08DA5F86B605}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5c50ed2d-852b-4196-83c6-52aa9500028d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5c50ed2d-852b-4196-83c6-52aa9500028d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93316912-AE26-426F-A937-08DA5F86B605}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>